<commit_message>
Seed a starter vocab list and CEFR level at signup
Signup now asks for a language pair (I already know / I'm learning)
and a CEFR level, reusing the existing Dropdown and CefrLevelPicker
components. Since /signup never returns a session (email confirmation
may be required), the actual seeding happens on this account's first
successful login instead: the chosen level becomes the device default,
and a 50-word starter vocab list is saved for the chosen language pair.

New src/lib/starter-vocab.ts holds the 50 concepts translated across
English/Spanish/French (same content as sample-vocab-lists' vocab-50
sets) so a starter list can be built for any pair among the three,
including pairs with no existing sample file (e.g. Spanish -> French).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3079,6 +3079,72 @@
       <c r="F122" s="5" t="inlineStr">
         <is>
           <t>Needs its own translation strategy — see Notes tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>login.tsx</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>starter_vocab_list_name</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>{language} Starter Vocab</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr">
+        <is>
+          <t>Auto-generated list name for the signup-seeded starter vocab list; template</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>login.tsx</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>i_already_know_reused</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>I already know</t>
+        </is>
+      </c>
+      <c r="F124" s="5" t="inlineStr">
+        <is>
+          <t>Reuses language-picker.tsx wording — shown in signup mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>login.tsx</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>i_am_learning_reused</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>I'm learning</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>Reuses language-picker.tsx wording — shown in signup mode</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace signup-time list seeding with a Sample Lists catalog
Reverted the signup screen back to plain email/password — collecting
one language pair at signup wrongly assumed a user only studies one
language. Instead, My Lists now has a "Sample Lists" section listing
every direction between the app's supported languages (6 pairs x
Vocab/Verbs = up to 12 entries, using starter-vocab.ts's existing data
plus new starter-verbs.ts), each addable independently and repeatedly
via the existing save-list endpoint (which already updates in place by
name, so re-adding is harmless).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3085,68 +3085,180 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>login.tsx</t>
+          <t>my-lists.tsx</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>starter_vocab_list_name</t>
+          <t>sample_lists_title</t>
         </is>
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>{language} Starter Vocab</t>
-        </is>
-      </c>
-      <c r="F123" s="5" t="inlineStr">
-        <is>
-          <t>Auto-generated list name for the signup-seeded starter vocab list; template</t>
-        </is>
-      </c>
+          <t>Sample Lists</t>
+        </is>
+      </c>
+      <c r="F123" s="5" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>login.tsx</t>
+          <t>my-lists.tsx</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>i_already_know_reused</t>
+          <t>sample_lists_hint</t>
         </is>
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>I already know</t>
-        </is>
-      </c>
-      <c r="F124" s="5" t="inlineStr">
-        <is>
-          <t>Reuses language-picker.tsx wording — shown in signup mode</t>
-        </is>
-      </c>
+          <t>Add a ready-made 50-word list for any language pair — add as many as you want, whenever you want.</t>
+        </is>
+      </c>
+      <c r="F124" s="5" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>login.tsx</t>
+          <t>my-lists.tsx</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>i_am_learning_reused</t>
+          <t>sample_list_name_template</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>I'm learning</t>
+          <t>{source} → {target} Vocab / {source} → {target} Verbs</t>
         </is>
       </c>
       <c r="F125" s="5" t="inlineStr">
         <is>
-          <t>Reuses language-picker.tsx wording — shown in signup mode</t>
-        </is>
-      </c>
+          <t>Template — used as both display label and saved list name</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_type_vocab</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>Vocab</t>
+        </is>
+      </c>
+      <c r="F126" s="5" t="inlineStr">
+        <is>
+          <t>Reused label under each sample list row</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_type_verbs</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>Verbs</t>
+        </is>
+      </c>
+      <c r="F127" s="5" t="inlineStr">
+        <is>
+          <t>Reused label under each sample list row</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_add</t>
+        </is>
+      </c>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="F128" s="5" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_adding</t>
+        </is>
+      </c>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>Adding…</t>
+        </is>
+      </c>
+      <c r="F129" s="5" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_added</t>
+        </is>
+      </c>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="F130" s="5" t="inlineStr">
+        <is>
+          <t>Shown once a list with the same name already exists; still tappable to re-sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>error_adding_sample</t>
+        </is>
+      </c>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>Something went wrong adding that sample list.</t>
+        </is>
+      </c>
+      <c r="F131" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add first-time onboarding (3 slides) and sync EAS-generated app.json
- New onboarding.tsx: 3-slide first-launch explainer (build a list /
  adaptive quizzes / progress tracking), simple inline SVG icons
  instead of screenshots (which go stale on every UI change), gated by
  a one-time SecureStore flag checked from Home. Replayable via a new
  "About LangReps" link in Settings.
- app.json now reflects the EAS build:configure output from the last
  few builds (iOS bundle identifier, export-compliance flag, EAS
  project id/owner, Android versionCode bump) — not committed until
  now.
- UI strings spreadsheet updated with the new onboarding/settings copy.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3259,6 +3259,208 @@
         </is>
       </c>
       <c r="F131" s="5" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>Skip</t>
+        </is>
+      </c>
+      <c r="F132" s="5" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>back</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>Back</t>
+        </is>
+      </c>
+      <c r="F133" s="5" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>next</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="F134" s="5" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>get_started</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>Get Started</t>
+        </is>
+      </c>
+      <c r="F135" s="5" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>slide1_headline</t>
+        </is>
+      </c>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>Build Your List</t>
+        </is>
+      </c>
+      <c r="F136" s="5" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>slide1_body</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Type words, paste a list, upload a file, or snap a photo — AI reads it for you. Or jump right in with a few ready-made sample lists in My Lists.</t>
+        </is>
+      </c>
+      <c r="F137" s="5" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>slide2_headline</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>Practice With Adaptive Quizzes</t>
+        </is>
+      </c>
+      <c r="F138" s="5" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>slide2_body</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>AI generates real sentences to test you — and the more you practice, the more it targets what you're actually struggling with.</t>
+        </is>
+      </c>
+      <c r="F139" s="5" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>slide3_headline</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Watch Your Progress</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>slide3_body</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>See your scores improve over time, list by list.</t>
+        </is>
+      </c>
+      <c r="F141" s="5" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>about_langreps_link</t>
+        </is>
+      </c>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>About LangReps</t>
+        </is>
+      </c>
+      <c r="F142" s="5" t="inlineStr">
+        <is>
+          <t>Links to /onboarding to replay it manually</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Clearer sample list names, last-uploaded date, and sortable My Lists
- Sample list names now read naturally ("Spanish Vocabulary (from
  English)") instead of the arrow-notation "English -> Spanish Vocab" —
  source language is kept in the name to avoid two entries (e.g.
  English->Spanish and French->Spanish) colliding, since save-list
  treats a repeated name as an update-in-place.
- Each saved list now shows a "Last uploaded" date (last_modified,
  already returned by GET /lists, just wasn't displayed).
- My Lists is now sortable by Date (most recent first, default) or
  Name.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F142"/>
+  <dimension ref="A1:F147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3459,6 +3459,104 @@
       <c r="F142" s="5" t="inlineStr">
         <is>
           <t>Links to /onboarding to replay it manually</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B143" s="3" t="inlineStr">
+        <is>
+          <t>sort_by_label</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>Sort by</t>
+        </is>
+      </c>
+      <c r="F143" s="5" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>sort_by_date</t>
+        </is>
+      </c>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="F144" s="5" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>sort_by_name</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="F145" s="5" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>last_uploaded_template</t>
+        </is>
+      </c>
+      <c r="C146" s="4" t="inlineStr">
+        <is>
+          <t>Last uploaded: {date}</t>
+        </is>
+      </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>Template — date formatting via toLocaleDateString(), varies by device locale</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_name_template_v2</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>{target} Vocabulary (from {source}) / {target} Verbs (from {source})</t>
+        </is>
+      </c>
+      <c r="F147" s="5" t="inlineStr">
+        <is>
+          <t>Superseded template — replaces the old arrow-notation naming</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use flag emoji + word count for Sample Lists cards
Replaces the spelled-out "Spanish Vocabulary (from English)" card
display with "Vocab 50" / flag -> flag — sidesteps the language-name
capitalization inconsistency entirely and reads faster when scanning
12 catalog entries. The underlying saved list name (used once actually
added, shown in Your Lists) is unchanged.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F147"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3557,6 +3557,50 @@
       <c r="F147" s="5" t="inlineStr">
         <is>
           <t>Superseded template — replaces the old arrow-notation naming</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_card_title</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>Vocab {count} / Verb {count}</t>
+        </is>
+      </c>
+      <c r="F148" s="5" t="inlineStr">
+        <is>
+          <t>Sample-list catalog card title, replaces the old full name display</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>sample_list_card_flags</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>{flag} -&gt; {flag}</t>
+        </is>
+      </c>
+      <c r="F149" s="5" t="inlineStr">
+        <is>
+          <t>Flag emoji pair instead of spelled-out language names — sidesteps capitalization inconsistency entirely</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add signup incentive hint, rename Share a Picture to Upload a Photo
- Home now shows a one-line hint under Log In/Sign Up explaining why
  it's worth doing (saving lists, tracking progress) — previously
  anonymous users had no indication their list disappears on close.
- "Share a Picture" was ambiguous (sharing to someone vs. uploading to
  the app) — renamed to "Upload a Photo" on Home and the screen itself,
  matching "Upload a File"'s naming pattern.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F149"/>
+  <dimension ref="A1:F150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -723,7 +723,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Share a Picture</t>
+          <t>Upload a Photo</t>
         </is>
       </c>
       <c r="D12" s="2" t="n"/>
@@ -1387,7 +1387,7 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Share a Picture</t>
+          <t>Upload a Photo</t>
         </is>
       </c>
       <c r="D43" s="2" t="n"/>
@@ -3603,6 +3603,24 @@
           <t>Flag emoji pair instead of spelled-out language names — sidesteps capitalization inconsistency entirely</t>
         </is>
       </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>index.tsx</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>signup_incentive_hint</t>
+        </is>
+      </c>
+      <c r="C150" s="4" t="inlineStr">
+        <is>
+          <t>Sign up to save your lists and track your progress over time</t>
+        </is>
+      </c>
+      <c r="F150" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Require Accents setting, restyle Settings, bulk-select delete for lists/quizzes
- New Settings toggle to grade answers exactly instead of stripping
  accents by default (app is a reinforcement tool, not a first-time
  teacher, so lenient grading stays the default).
- Settings screen now shows a bold title + description per option
  instead of one dense hint line.
- My Lists and My Quizzes both gain a "Select" mode: checkboxes,
  Select All/Deselect All, and a single "Delete Selected" bulk action,
  so testers aren't stuck deleting saved lists/quizzes one at a time.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="UI Strings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legend" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,41 +26,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00808080"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
-        <bgColor rgb="002F5496"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -76,20 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,11 +417,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:G167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
@@ -499,3218 +461,3587 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>app_name</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>LangReps</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
         <is>
           <t>Proper name — may stay untranslated</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>home_subtitle</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Build a vocab list, then let AI generate an adaptive quiz for it.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>settings_link</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Settings</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>log_out</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Log Out</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>delete_account</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Delete Account</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Also used as alert title</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>log_in_sign_up</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Log In / Sign Up</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>signed_in_as</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Signed in as {email}</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
         <is>
           <t>Template — {email} not translated</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>add_words_manually</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Add Words Manually</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>paste_vocab_list</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Paste Vocab List</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="5" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>upload_a_file</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Upload a File</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="5" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>share_a_picture</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Upload a Photo</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="5" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>my_lists</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>My Lists</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="5" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>my_quizzes</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>My Quizzes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="5" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>delete_account_confirm</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>This permanently deletes your account and all your saved lists. This can't be undone.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
         <is>
           <t>Alert body</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>cancel</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Cancel</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
         <is>
           <t>Alert button — reused across screens</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>delete</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Delete</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
         <is>
           <t>Alert button — reused across screens</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>error_generic</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Something went wrong.</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
         <is>
           <t>Fallback error — reused across screens</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>log_in</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Log In</t>
         </is>
       </c>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
         <is>
           <t>Screen title + button + toggle target</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>sign_up</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Sign Up</t>
         </is>
       </c>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
         <is>
           <t>Screen title + button + toggle target</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>email_placeholder</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="5" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>password_placeholder</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="5" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>please_wait</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Please wait…</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="5" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>switch_to_signup</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Don't have an account? Sign up</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="5" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>switch_to_login</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Already have an account? Log in</t>
         </is>
       </c>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="5" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>confirm_email_message</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Check your email to confirm, then log in below.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="5" t="inlineStr"/>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>login.tsx</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>account_created_message</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Account created — log in below.</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="5" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>add-words.tsx</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>add_words_title</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Add Words</t>
         </is>
       </c>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="5" t="inlineStr"/>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>add-words.tsx</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>source_word_placeholder</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Source word</t>
         </is>
       </c>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="2" t="n"/>
-      <c r="F29" s="5" t="inlineStr"/>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>add-words.tsx</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>target_word_placeholder</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>Target word</t>
         </is>
       </c>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="5" t="inlineStr"/>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>add-words.tsx</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>add_to_list</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Add to list</t>
         </is>
       </c>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
         <is>
           <t>Reused on paste-text.tsx</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>paste-text.tsx</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>paste_vocab_list_title</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>Paste Vocab List</t>
         </is>
       </c>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="5" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>paste-text.tsx</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>paste_instructions</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>One pair per line — a tab, "-&gt;", ":", or similar between each word and its translation. e.g. hello -&gt; hola</t>
         </is>
       </c>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="2" t="n"/>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
         <is>
           <t>Contains a literal example — keep example untranslated or localize it</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>paste-text.tsx</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>paste_placeholder</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Paste your vocab list here</t>
         </is>
       </c>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="5" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>paste-text.tsx</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>parsing_ellipsis</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Parsing…</t>
         </is>
       </c>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
         <is>
           <t>Reused on upload-file.tsx</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>paste-text.tsx</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>couldnt_parse_lines</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>Couldn't parse {n} line(s): {list}</t>
         </is>
       </c>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="5" t="inlineStr">
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
         <is>
           <t>Template with pluralization (1 line vs N lines)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>paste-text.tsx</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>error_parsing_text</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>Something went wrong parsing that text.</t>
         </is>
       </c>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="5" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>upload-file.tsx</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>upload_a_file_title</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>Upload a File</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="5" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>upload-file.tsx</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>upload_file_instructions</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>A plain text or CSV file, one pair per line — a tab, "-&gt;", ":", or similar between each word and its translation.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="5" t="inlineStr"/>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>upload-file.tsx</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>choose_file</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Choose File</t>
         </is>
       </c>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="5" t="inlineStr"/>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>upload-file.tsx</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>last_file</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>Last file: {name}</t>
         </is>
       </c>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
         <is>
           <t>Template — filename not translated</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>upload-file.tsx</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>error_parsing_file</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>Something went wrong parsing that file.</t>
         </is>
       </c>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>share_a_picture_title</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>Upload a Photo</t>
         </is>
       </c>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="5" t="inlineStr"/>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>share_picture_instructions</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>A photo or screenshot of word pairs (e.g. "house -&gt; casa") — AI will read the pairs out of it.</t>
         </is>
       </c>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="5" t="inlineStr">
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
         <is>
           <t>Contains a literal example</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>take_photo</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>Take Photo</t>
         </is>
       </c>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="2" t="n"/>
-      <c r="F45" s="5" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>choose_from_library</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>Choose from Library</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="5" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>reading_ellipsis</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>Reading…</t>
         </is>
       </c>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="2" t="n"/>
-      <c r="F47" s="5" t="inlineStr"/>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>error_camera_permission</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Camera access is needed to take a photo.</t>
         </is>
       </c>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="2" t="n"/>
-      <c r="F48" s="5" t="inlineStr"/>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>error_library_permission</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Photo library access is needed to choose an image.</t>
         </is>
       </c>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="2" t="n"/>
-      <c r="F49" s="5" t="inlineStr"/>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>upload-picture.tsx</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>error_reading_image</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>Something went wrong reading that image.</t>
         </is>
       </c>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="5" t="inlineStr"/>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>generate_quiz_title</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>Generate Quiz</t>
         </is>
       </c>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="2" t="n"/>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
         <is>
           <t>Also reused as button label</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>unsaved_list</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>Unsaved list</t>
         </is>
       </c>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
         <is>
           <t>Fallback when no list name</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>min_words_warning</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>You need at least 3 words to generate a quiz.</t>
         </is>
       </c>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="2" t="n"/>
-      <c r="F53" s="5" t="inlineStr"/>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>words_in_list</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>{n} words in this list.</t>
         </is>
       </c>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="5" t="inlineStr">
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
         <is>
           <t>Template with pluralization</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>how_many_questions</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>How many questions?</t>
         </is>
       </c>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="2" t="n"/>
-      <c r="F55" s="5" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>tense_label</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>Tense</t>
         </is>
       </c>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="2" t="n"/>
-      <c r="F56" s="5" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>mixed_tense</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Mixed</t>
         </is>
       </c>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="2" t="n"/>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
         <is>
           <t>Dropdown option meaning vary tense freely</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>flip_toggle_label</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>Flip: translate {target} → {source}</t>
         </is>
       </c>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="2" t="n"/>
-      <c r="F58" s="5" t="inlineStr">
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
         <is>
           <t>Template — language names not translated here</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>generating_quiz</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Generating your quiz…</t>
         </is>
       </c>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="2" t="n"/>
-      <c r="F59" s="5" t="inlineStr"/>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="A60" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>target_my_mistakes</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>Target My Mistakes</t>
         </is>
       </c>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="2" t="n"/>
-      <c r="F60" s="5" t="inlineStr"/>
+      <c r="D60" t="inlineStr"/>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>generate_similar_quiz</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>Generate Similar Quiz</t>
         </is>
       </c>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="2" t="n"/>
-      <c r="F61" s="5" t="inlineStr"/>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="A62" t="inlineStr">
         <is>
           <t>generate-quiz.tsx</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>error_generating_quiz</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>Something went wrong generating your quiz.</t>
         </is>
       </c>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="n"/>
-      <c r="F62" s="5" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="A63" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>my_lists_title</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>My Lists</t>
         </is>
       </c>
-      <c r="D63" s="2" t="n"/>
-      <c r="E63" s="2" t="n"/>
-      <c r="F63" s="5" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="A64" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>no_saved_lists</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>No saved lists yet.</t>
         </is>
       </c>
-      <c r="D64" s="2" t="n"/>
-      <c r="E64" s="2" t="n"/>
-      <c r="F64" s="5" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="A65" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>progress_link</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="2" t="n"/>
-      <c r="F65" s="5" t="inlineStr">
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
         <is>
           <t>Row action label</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>delete_list_alert_title</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>Delete List</t>
         </is>
       </c>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="5" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>delete_list_confirm</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>Delete "{name}"? This can't be undone.</t>
         </is>
       </c>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
-      <c r="F67" s="5" t="inlineStr">
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>error_loading_lists</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>Something went wrong loading your lists.</t>
         </is>
       </c>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="2" t="n"/>
-      <c r="F68" s="5" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>error_loading_list</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>Something went wrong loading that list.</t>
         </is>
       </c>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
-      <c r="F69" s="5" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>error_deleting_list</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>Something went wrong deleting that list.</t>
         </is>
       </c>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="n"/>
-      <c r="F70" s="5" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>my_quizzes_title</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>My Quizzes</t>
         </is>
       </c>
-      <c r="D71" s="2" t="n"/>
-      <c r="E71" s="2" t="n"/>
-      <c r="F71" s="5" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="inlineStr">
+      <c r="A72" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>no_quizzes_in_progress</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>No quizzes in progress.</t>
         </is>
       </c>
-      <c r="D72" s="2" t="n"/>
-      <c r="E72" s="2" t="n"/>
-      <c r="F72" s="5" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="inlineStr">
+      <c r="A73" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>quiz_in_progress_fallback</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Quiz in progress</t>
         </is>
       </c>
-      <c r="D73" s="2" t="n"/>
-      <c r="E73" s="2" t="n"/>
-      <c r="F73" s="5" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
+      <c r="A74" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>question_n_of_total</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>Question {n} of {total}</t>
         </is>
       </c>
-      <c r="D74" s="2" t="n"/>
-      <c r="E74" s="2" t="n"/>
-      <c r="F74" s="5" t="inlineStr">
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
         <is>
           <t>Template — also used in quiz.tsx</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+      <c r="A75" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>delete_quiz_alert_title</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>Delete Quiz</t>
         </is>
       </c>
-      <c r="D75" s="2" t="n"/>
-      <c r="E75" s="2" t="n"/>
-      <c r="F75" s="5" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+      <c r="A76" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>delete_quiz_confirm</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>Delete this quiz for "{name}"? This can't be undone.</t>
         </is>
       </c>
-      <c r="D76" s="2" t="n"/>
-      <c r="E76" s="2" t="n"/>
-      <c r="F76" s="5" t="inlineStr">
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="A77" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>error_loading_quizzes</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>Something went wrong loading your quizzes.</t>
         </is>
       </c>
-      <c r="D77" s="2" t="n"/>
-      <c r="E77" s="2" t="n"/>
-      <c r="F77" s="5" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="A78" t="inlineStr">
         <is>
           <t>my-quizzes.tsx</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>error_deleting_quiz</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>Something went wrong deleting that quiz.</t>
         </is>
       </c>
-      <c r="D78" s="2" t="n"/>
-      <c r="E78" s="2" t="n"/>
-      <c r="F78" s="5" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+      <c r="A79" t="inlineStr">
         <is>
           <t>list-history.tsx</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>progress_title</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>Progress</t>
         </is>
       </c>
-      <c r="D79" s="2" t="n"/>
-      <c r="E79" s="2" t="n"/>
-      <c r="F79" s="5" t="inlineStr">
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr">
         <is>
           <t>Title fallback + subtitle label</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="A80" t="inlineStr">
         <is>
           <t>list-history.tsx</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>no_completed_quizzes</t>
         </is>
       </c>
-      <c r="C80" s="4" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>No completed quizzes for this list yet.</t>
         </is>
       </c>
-      <c r="D80" s="2" t="n"/>
-      <c r="E80" s="2" t="n"/>
-      <c r="F80" s="5" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="inlineStr">
+      <c r="A81" t="inlineStr">
         <is>
           <t>list-history.tsx</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>score_fraction_pct</t>
         </is>
       </c>
-      <c r="C81" s="4" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>{correct}/{total} ({pct}%)</t>
         </is>
       </c>
-      <c r="D81" s="2" t="n"/>
-      <c r="E81" s="2" t="n"/>
-      <c r="F81" s="5" t="inlineStr">
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
         <is>
           <t>Number formatting conventions vary by locale</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="A82" t="inlineStr">
         <is>
           <t>list-history.tsx</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>error_loading_history</t>
         </is>
       </c>
-      <c r="C82" s="4" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>Something went wrong loading quiz history.</t>
         </is>
       </c>
-      <c r="D82" s="2" t="n"/>
-      <c r="E82" s="2" t="n"/>
-      <c r="F82" s="5" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
+      <c r="A83" t="inlineStr">
         <is>
           <t>settings.tsx</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>settings_title</t>
         </is>
       </c>
-      <c r="C83" s="4" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>Settings</t>
         </is>
       </c>
-      <c r="D83" s="2" t="n"/>
-      <c r="E83" s="2" t="n"/>
-      <c r="F83" s="5" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
+      <c r="A84" t="inlineStr">
         <is>
           <t>settings.tsx</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>default_level_hint</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Default level for new quizzes — you can still change it for any single quiz when generating it.</t>
         </is>
       </c>
-      <c r="D84" s="2" t="n"/>
-      <c r="E84" s="2" t="n"/>
-      <c r="F84" s="5" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+      <c r="A85" t="inlineStr">
         <is>
           <t>settings.tsx</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>auto_delete_toggle</t>
         </is>
       </c>
-      <c r="C85" s="4" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Auto-delete completed quizzes after 30 days</t>
         </is>
       </c>
-      <c r="D85" s="2" t="n"/>
-      <c r="E85" s="2" t="n"/>
-      <c r="F85" s="5" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr">
+      <c r="A86" t="inlineStr">
         <is>
           <t>settings.tsx</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>adaptive_quizzes_toggle</t>
         </is>
       </c>
-      <c r="C86" s="4" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>Adaptive quizzes — feedback on patterns you struggle with, and an option to target them</t>
         </is>
       </c>
-      <c r="D86" s="2" t="n"/>
-      <c r="E86" s="2" t="n"/>
-      <c r="F86" s="5" t="inlineStr"/>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
+      <c r="A87" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B87" s="3" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>your_answer_placeholder</t>
         </is>
       </c>
-      <c r="C87" s="4" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>Your answer</t>
         </is>
       </c>
-      <c r="D87" s="2" t="n"/>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="5" t="inlineStr"/>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="inlineStr">
+      <c r="A88" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>submit</t>
         </is>
       </c>
-      <c r="C88" s="4" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Submit</t>
         </is>
       </c>
-      <c r="D88" s="2" t="n"/>
-      <c r="E88" s="2" t="n"/>
-      <c r="F88" s="5" t="inlineStr"/>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="inlineStr">
+      <c r="A89" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B89" s="3" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>skip_question</t>
         </is>
       </c>
-      <c r="C89" s="4" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>Skip this question</t>
         </is>
       </c>
-      <c r="D89" s="2" t="n"/>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="5" t="inlineStr"/>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr">
+      <c r="A90" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>hide_word_list</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>Hide word list</t>
         </is>
       </c>
-      <c r="D90" s="2" t="n"/>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="5" t="inlineStr"/>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr">
+      <c r="A91" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>stuck_see_word_list</t>
         </is>
       </c>
-      <c r="C91" s="4" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>Stuck? See the word list</t>
         </is>
       </c>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="n"/>
-      <c r="F91" s="5" t="inlineStr"/>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="inlineStr">
+      <c r="A92" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B92" s="3" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>your_answer_was</t>
         </is>
       </c>
-      <c r="C92" s="4" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>Your answer: {answer}</t>
         </is>
       </c>
-      <c r="D92" s="2" t="n"/>
-      <c r="E92" s="2" t="n"/>
-      <c r="F92" s="5" t="inlineStr">
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+      <c r="A93" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>correct_feedback</t>
         </is>
       </c>
-      <c r="C93" s="4" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>That's correct!</t>
         </is>
       </c>
-      <c r="D93" s="2" t="n"/>
-      <c r="E93" s="2" t="n"/>
-      <c r="F93" s="5" t="inlineStr"/>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr">
+      <c r="A94" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B94" s="3" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>incorrect_feedback</t>
         </is>
       </c>
-      <c r="C94" s="4" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>Sorry, that's incorrect. The answer was: {answer}</t>
         </is>
       </c>
-      <c r="D94" s="2" t="n"/>
-      <c r="E94" s="2" t="n"/>
-      <c r="F94" s="5" t="inlineStr">
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="inlineStr">
+      <c r="A95" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B95" s="3" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>finish_quiz</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Finish Quiz</t>
         </is>
       </c>
-      <c r="D95" s="2" t="n"/>
-      <c r="E95" s="2" t="n"/>
-      <c r="F95" s="5" t="inlineStr"/>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr">
+      <c r="A96" t="inlineStr">
         <is>
           <t>quiz.tsx</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>next_question</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>Next Question</t>
         </is>
       </c>
-      <c r="D96" s="2" t="n"/>
-      <c r="E96" s="2" t="n"/>
-      <c r="F96" s="5" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="inlineStr">
+      <c r="A97" t="inlineStr">
         <is>
           <t>quiz-complete.tsx</t>
         </is>
       </c>
-      <c r="B97" s="3" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>quiz_complete_title</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>Quiz Complete!</t>
         </is>
       </c>
-      <c r="D97" s="2" t="n"/>
-      <c r="E97" s="2" t="n"/>
-      <c r="F97" s="5" t="inlineStr"/>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="inlineStr">
+      <c r="A98" t="inlineStr">
         <is>
           <t>quiz-complete.tsx</t>
         </is>
       </c>
-      <c r="B98" s="3" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>score_correct</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>{n} / {total} correct</t>
         </is>
       </c>
-      <c r="D98" s="2" t="n"/>
-      <c r="E98" s="2" t="n"/>
-      <c r="F98" s="5" t="inlineStr">
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr">
         <is>
           <t>Template</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="inlineStr">
+      <c r="A99" t="inlineStr">
         <is>
           <t>quiz-complete.tsx</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>back_to_home</t>
         </is>
       </c>
-      <c r="C99" s="4" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>Back to Home</t>
         </is>
       </c>
-      <c r="D99" s="2" t="n"/>
-      <c r="E99" s="2" t="n"/>
-      <c r="F99" s="5" t="inlineStr"/>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
+      <c r="A100" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B100" s="3" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>undo_last</t>
         </is>
       </c>
-      <c r="C100" s="4" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>Undo last</t>
         </is>
       </c>
-      <c r="D100" s="2" t="n"/>
-      <c r="E100" s="2" t="n"/>
-      <c r="F100" s="5" t="inlineStr"/>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="inlineStr">
+      <c r="A101" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B101" s="3" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>clear_list</t>
         </is>
       </c>
-      <c r="C101" s="4" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>Clear list</t>
         </is>
       </c>
-      <c r="D101" s="2" t="n"/>
-      <c r="E101" s="2" t="n"/>
-      <c r="F101" s="5" t="inlineStr"/>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr">
+      <c r="A102" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B102" s="3" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>no_words_added</t>
         </is>
       </c>
-      <c r="C102" s="4" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>No words added yet.</t>
         </is>
       </c>
-      <c r="D102" s="2" t="n"/>
-      <c r="E102" s="2" t="n"/>
-      <c r="F102" s="5" t="inlineStr"/>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="inlineStr">
+      <c r="A103" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>list_name_update_placeholder</t>
         </is>
       </c>
-      <c r="C103" s="4" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>List name (saving updates it)</t>
         </is>
       </c>
-      <c r="D103" s="2" t="n"/>
-      <c r="E103" s="2" t="n"/>
-      <c r="F103" s="5" t="inlineStr"/>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="inlineStr">
+      <c r="A104" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B104" s="3" t="inlineStr">
+      <c r="B104" t="inlineStr">
         <is>
           <t>list_name_placeholder</t>
         </is>
       </c>
-      <c r="C104" s="4" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>List name</t>
         </is>
       </c>
-      <c r="D104" s="2" t="n"/>
-      <c r="E104" s="2" t="n"/>
-      <c r="F104" s="5" t="inlineStr"/>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="inlineStr">
+      <c r="A105" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B105" s="3" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>saving_ellipsis</t>
         </is>
       </c>
-      <c r="C105" s="4" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>Saving…</t>
         </is>
       </c>
-      <c r="D105" s="2" t="n"/>
-      <c r="E105" s="2" t="n"/>
-      <c r="F105" s="5" t="inlineStr"/>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="inlineStr">
+      <c r="A106" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B106" s="3" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>save_list</t>
         </is>
       </c>
-      <c r="C106" s="4" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>Save List</t>
         </is>
       </c>
-      <c r="D106" s="2" t="n"/>
-      <c r="E106" s="2" t="n"/>
-      <c r="F106" s="5" t="inlineStr"/>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
+      <c r="A107" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B107" s="3" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>saved_message</t>
         </is>
       </c>
-      <c r="C107" s="4" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>Saved!</t>
         </is>
       </c>
-      <c r="D107" s="2" t="n"/>
-      <c r="E107" s="2" t="n"/>
-      <c r="F107" s="5" t="inlineStr"/>
+      <c r="D107" t="inlineStr"/>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
+      <c r="A108" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B108" s="3" t="inlineStr">
+      <c r="B108" t="inlineStr">
         <is>
           <t>error_saving</t>
         </is>
       </c>
-      <c r="C108" s="4" t="inlineStr">
+      <c r="C108" t="inlineStr">
         <is>
           <t>Something went wrong saving.</t>
         </is>
       </c>
-      <c r="D108" s="2" t="n"/>
-      <c r="E108" s="2" t="n"/>
-      <c r="F108" s="5" t="inlineStr"/>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="inlineStr">
+      <c r="A109" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B109" s="3" t="inlineStr">
+      <c r="B109" t="inlineStr">
         <is>
           <t>add_more_words_to_quiz</t>
         </is>
       </c>
-      <c r="C109" s="4" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>Add {n} more word(s) to generate a quiz</t>
         </is>
       </c>
-      <c r="D109" s="2" t="n"/>
-      <c r="E109" s="2" t="n"/>
-      <c r="F109" s="5" t="inlineStr">
+      <c r="D109" t="inlineStr"/>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr">
         <is>
           <t>Template with pluralization</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="inlineStr">
+      <c r="A110" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>generate_quiz_button</t>
         </is>
       </c>
-      <c r="C110" s="4" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>Generate Quiz</t>
         </is>
       </c>
-      <c r="D110" s="2" t="n"/>
-      <c r="E110" s="2" t="n"/>
-      <c r="F110" s="5" t="inlineStr">
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr">
         <is>
           <t>Reused label</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="inlineStr">
+      <c r="A111" t="inlineStr">
         <is>
           <t>pairs-review.tsx</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>my_lists_link</t>
         </is>
       </c>
-      <c r="C111" s="4" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>My Lists</t>
         </is>
       </c>
-      <c r="D111" s="2" t="n"/>
-      <c r="E111" s="2" t="n"/>
-      <c r="F111" s="5" t="inlineStr">
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
         <is>
           <t>Reused label</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="inlineStr">
+      <c r="A112" t="inlineStr">
         <is>
           <t>cefr-level-picker.tsx</t>
         </is>
       </c>
-      <c r="B112" s="3" t="inlineStr">
+      <c r="B112" t="inlineStr">
         <is>
           <t>level_label</t>
         </is>
       </c>
-      <c r="C112" s="4" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="D112" s="2" t="n"/>
-      <c r="E112" s="2" t="n"/>
-      <c r="F112" s="5" t="inlineStr">
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
         <is>
           <t>CEFR codes (A1, B2, etc.) are standard notation, not translated</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="inlineStr">
+      <c r="A113" t="inlineStr">
         <is>
           <t>language-picker.tsx</t>
         </is>
       </c>
-      <c r="B113" s="3" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>i_already_know</t>
         </is>
       </c>
-      <c r="C113" s="4" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>I already know</t>
         </is>
       </c>
-      <c r="D113" s="2" t="n"/>
-      <c r="E113" s="2" t="n"/>
-      <c r="F113" s="5" t="inlineStr"/>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr">
+      <c r="A114" t="inlineStr">
         <is>
           <t>language-picker.tsx</t>
         </is>
       </c>
-      <c r="B114" s="3" t="inlineStr">
+      <c r="B114" t="inlineStr">
         <is>
           <t>i_am_learning</t>
         </is>
       </c>
-      <c r="C114" s="4" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t>I'm learning</t>
         </is>
       </c>
-      <c r="D114" s="2" t="n"/>
-      <c r="E114" s="2" t="n"/>
-      <c r="F114" s="5" t="inlineStr"/>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="inlineStr">
+      <c r="A115" t="inlineStr">
         <is>
           <t>language-picker.tsx</t>
         </is>
       </c>
-      <c r="B115" s="3" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>language_names</t>
         </is>
       </c>
-      <c r="C115" s="4" t="inlineStr">
+      <c r="C115" t="inlineStr">
         <is>
           <t>English / Spanish / French</t>
         </is>
       </c>
-      <c r="D115" s="2" t="n"/>
-      <c r="E115" s="2" t="n"/>
-      <c r="F115" s="5" t="inlineStr">
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
         <is>
           <t>Design decision: show in UI language or always native form (Español, Français)?</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr">
+      <c r="A116" t="inlineStr">
         <is>
           <t>parsing-warning.tsx</t>
         </is>
       </c>
-      <c r="B116" s="3" t="inlineStr">
+      <c r="B116" t="inlineStr">
         <is>
           <t>parsing_warning_text</t>
         </is>
       </c>
-      <c r="C116" s="4" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>Parsing can make mistakes with unusual formatting. For best results, try Share a Picture instead.</t>
         </is>
       </c>
-      <c r="D116" s="2" t="n"/>
-      <c r="E116" s="2" t="n"/>
-      <c r="F116" s="5" t="inlineStr">
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
         <is>
           <t>Contains an inline link to Share a Picture</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="inlineStr">
+      <c r="A117" t="inlineStr">
         <is>
           <t>quiz-feedback.ts</t>
         </is>
       </c>
-      <c r="B117" s="3" t="inlineStr">
+      <c r="B117" t="inlineStr">
         <is>
           <t>trend_improving_a_lot</t>
         </is>
       </c>
-      <c r="C117" s="4" t="inlineStr">
+      <c r="C117" t="inlineStr">
         <is>
           <t>5 message variants — 'Great progress! Your scores are climbing fast...' etc.</t>
         </is>
       </c>
-      <c r="D117" s="2" t="n"/>
-      <c r="E117" s="2" t="n"/>
-      <c r="F117" s="5" t="inlineStr">
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
         <is>
           <t>See file directly, too long to list individually</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="inlineStr">
+      <c r="A118" t="inlineStr">
         <is>
           <t>quiz-feedback.ts</t>
         </is>
       </c>
-      <c r="B118" s="3" t="inlineStr">
+      <c r="B118" t="inlineStr">
         <is>
           <t>trend_improving</t>
         </is>
       </c>
-      <c r="C118" s="4" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>5 message variants — 'You're improving steadily on this list.' etc.</t>
         </is>
       </c>
-      <c r="D118" s="2" t="n"/>
-      <c r="E118" s="2" t="n"/>
-      <c r="F118" s="5" t="inlineStr">
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
         <is>
           <t>See file directly</t>
         </is>
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="inlineStr">
+      <c r="A119" t="inlineStr">
         <is>
           <t>quiz-feedback.ts</t>
         </is>
       </c>
-      <c r="B119" s="3" t="inlineStr">
+      <c r="B119" t="inlineStr">
         <is>
           <t>trend_steady</t>
         </is>
       </c>
-      <c r="C119" s="4" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>5 message variants — 'Your scores are holding steady...' etc.</t>
         </is>
       </c>
-      <c r="D119" s="2" t="n"/>
-      <c r="E119" s="2" t="n"/>
-      <c r="F119" s="5" t="inlineStr">
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
         <is>
           <t>See file directly</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="inlineStr">
+      <c r="A120" t="inlineStr">
         <is>
           <t>quiz-feedback.ts</t>
         </is>
       </c>
-      <c r="B120" s="3" t="inlineStr">
+      <c r="B120" t="inlineStr">
         <is>
           <t>trend_declining</t>
         </is>
       </c>
-      <c r="C120" s="4" t="inlineStr">
+      <c r="C120" t="inlineStr">
         <is>
           <t>5 message variants — 'Your scores dipped a bit recently...' etc.</t>
         </is>
       </c>
-      <c r="D120" s="2" t="n"/>
-      <c r="E120" s="2" t="n"/>
-      <c r="F120" s="5" t="inlineStr">
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
         <is>
           <t>See file directly</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="inlineStr">
+      <c r="A121" t="inlineStr">
         <is>
           <t>quiz-feedback.ts</t>
         </is>
       </c>
-      <c r="B121" s="3" t="inlineStr">
+      <c r="B121" t="inlineStr">
         <is>
           <t>trend_declining_a_lot</t>
         </is>
       </c>
-      <c r="C121" s="4" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>5 message variants — 'Your scores dropped noticeably...' etc.</t>
         </is>
       </c>
-      <c r="D121" s="2" t="n"/>
-      <c r="E121" s="2" t="n"/>
-      <c r="F121" s="5" t="inlineStr">
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
         <is>
           <t>See file directly</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="inlineStr">
+      <c r="A122" t="inlineStr">
         <is>
           <t>backend (api errors)</t>
         </is>
       </c>
-      <c r="B122" s="3" t="inlineStr">
+      <c r="B122" t="inlineStr">
         <is>
           <t>backend_error_text</t>
         </is>
       </c>
-      <c r="C122" s="4" t="inlineStr">
+      <c r="C122" t="inlineStr">
         <is>
           <t>Various FastAPI HTTPException / Pydantic validation messages surfaced via e.message</t>
         </is>
       </c>
-      <c r="D122" s="2" t="n"/>
-      <c r="E122" s="2" t="n"/>
-      <c r="F122" s="5" t="inlineStr">
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
         <is>
           <t>Needs its own translation strategy — see Notes tab</t>
         </is>
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="inlineStr">
+      <c r="A123" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B123" s="3" t="inlineStr">
+      <c r="B123" t="inlineStr">
         <is>
           <t>sample_lists_title</t>
         </is>
       </c>
-      <c r="C123" s="4" t="inlineStr">
+      <c r="C123" t="inlineStr">
         <is>
           <t>Sample Lists</t>
         </is>
       </c>
-      <c r="F123" s="5" t="inlineStr"/>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="inlineStr">
+      <c r="A124" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B124" s="3" t="inlineStr">
+      <c r="B124" t="inlineStr">
         <is>
           <t>sample_lists_hint</t>
         </is>
       </c>
-      <c r="C124" s="4" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>Add a ready-made 50-word list for any language pair — add as many as you want, whenever you want.</t>
         </is>
       </c>
-      <c r="F124" s="5" t="inlineStr"/>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="inlineStr">
+      <c r="A125" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B125" s="3" t="inlineStr">
+      <c r="B125" t="inlineStr">
         <is>
           <t>sample_list_name_template</t>
         </is>
       </c>
-      <c r="C125" s="4" t="inlineStr">
+      <c r="C125" t="inlineStr">
         <is>
           <t>{source} → {target} Vocab / {source} → {target} Verbs</t>
         </is>
       </c>
-      <c r="F125" s="5" t="inlineStr">
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
         <is>
           <t>Template — used as both display label and saved list name</t>
         </is>
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="inlineStr">
+      <c r="A126" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B126" s="3" t="inlineStr">
+      <c r="B126" t="inlineStr">
         <is>
           <t>sample_list_type_vocab</t>
         </is>
       </c>
-      <c r="C126" s="4" t="inlineStr">
+      <c r="C126" t="inlineStr">
         <is>
           <t>Vocab</t>
         </is>
       </c>
-      <c r="F126" s="5" t="inlineStr">
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
         <is>
           <t>Reused label under each sample list row</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="inlineStr">
+      <c r="A127" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B127" s="3" t="inlineStr">
+      <c r="B127" t="inlineStr">
         <is>
           <t>sample_list_type_verbs</t>
         </is>
       </c>
-      <c r="C127" s="4" t="inlineStr">
+      <c r="C127" t="inlineStr">
         <is>
           <t>Verbs</t>
         </is>
       </c>
-      <c r="F127" s="5" t="inlineStr">
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
         <is>
           <t>Reused label under each sample list row</t>
         </is>
       </c>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="inlineStr">
+      <c r="A128" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B128" s="3" t="inlineStr">
+      <c r="B128" t="inlineStr">
         <is>
           <t>sample_list_add</t>
         </is>
       </c>
-      <c r="C128" s="4" t="inlineStr">
+      <c r="C128" t="inlineStr">
         <is>
           <t>Add</t>
         </is>
       </c>
-      <c r="F128" s="5" t="inlineStr"/>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="inlineStr">
+      <c r="A129" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B129" s="3" t="inlineStr">
+      <c r="B129" t="inlineStr">
         <is>
           <t>sample_list_adding</t>
         </is>
       </c>
-      <c r="C129" s="4" t="inlineStr">
+      <c r="C129" t="inlineStr">
         <is>
           <t>Adding…</t>
         </is>
       </c>
-      <c r="F129" s="5" t="inlineStr"/>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="inlineStr">
+      <c r="A130" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B130" s="3" t="inlineStr">
+      <c r="B130" t="inlineStr">
         <is>
           <t>sample_list_added</t>
         </is>
       </c>
-      <c r="C130" s="4" t="inlineStr">
+      <c r="C130" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
       </c>
-      <c r="F130" s="5" t="inlineStr">
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
         <is>
           <t>Shown once a list with the same name already exists; still tappable to re-sync</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="inlineStr">
+      <c r="A131" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B131" s="3" t="inlineStr">
+      <c r="B131" t="inlineStr">
         <is>
           <t>error_adding_sample</t>
         </is>
       </c>
-      <c r="C131" s="4" t="inlineStr">
+      <c r="C131" t="inlineStr">
         <is>
           <t>Something went wrong adding that sample list.</t>
         </is>
       </c>
-      <c r="F131" s="5" t="inlineStr"/>
+      <c r="D131" t="inlineStr"/>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="inlineStr">
+      <c r="A132" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B132" s="3" t="inlineStr">
+      <c r="B132" t="inlineStr">
         <is>
           <t>skip</t>
         </is>
       </c>
-      <c r="C132" s="4" t="inlineStr">
+      <c r="C132" t="inlineStr">
         <is>
           <t>Skip</t>
         </is>
       </c>
-      <c r="F132" s="5" t="inlineStr"/>
+      <c r="D132" t="inlineStr"/>
+      <c r="E132" t="inlineStr"/>
+      <c r="F132" t="inlineStr"/>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="inlineStr">
+      <c r="A133" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B133" s="3" t="inlineStr">
+      <c r="B133" t="inlineStr">
         <is>
           <t>back</t>
         </is>
       </c>
-      <c r="C133" s="4" t="inlineStr">
+      <c r="C133" t="inlineStr">
         <is>
           <t>Back</t>
         </is>
       </c>
-      <c r="F133" s="5" t="inlineStr"/>
+      <c r="D133" t="inlineStr"/>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="inlineStr">
+      <c r="A134" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B134" s="3" t="inlineStr">
+      <c r="B134" t="inlineStr">
         <is>
           <t>next</t>
         </is>
       </c>
-      <c r="C134" s="4" t="inlineStr">
+      <c r="C134" t="inlineStr">
         <is>
           <t>Next</t>
         </is>
       </c>
-      <c r="F134" s="5" t="inlineStr"/>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="inlineStr">
+      <c r="A135" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B135" s="3" t="inlineStr">
+      <c r="B135" t="inlineStr">
         <is>
           <t>get_started</t>
         </is>
       </c>
-      <c r="C135" s="4" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>Get Started</t>
         </is>
       </c>
-      <c r="F135" s="5" t="inlineStr"/>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="inlineStr">
+      <c r="A136" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B136" s="3" t="inlineStr">
+      <c r="B136" t="inlineStr">
         <is>
           <t>slide1_headline</t>
         </is>
       </c>
-      <c r="C136" s="4" t="inlineStr">
+      <c r="C136" t="inlineStr">
         <is>
           <t>Build Your List</t>
         </is>
       </c>
-      <c r="F136" s="5" t="inlineStr"/>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="inlineStr">
+      <c r="A137" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B137" s="3" t="inlineStr">
+      <c r="B137" t="inlineStr">
         <is>
           <t>slide1_body</t>
         </is>
       </c>
-      <c r="C137" s="4" t="inlineStr">
+      <c r="C137" t="inlineStr">
         <is>
           <t>Type words, paste a list, upload a file, or snap a photo — AI reads it for you. Or jump right in with a few ready-made sample lists in My Lists.</t>
         </is>
       </c>
-      <c r="F137" s="5" t="inlineStr"/>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="inlineStr">
+      <c r="A138" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B138" s="3" t="inlineStr">
+      <c r="B138" t="inlineStr">
         <is>
           <t>slide2_headline</t>
         </is>
       </c>
-      <c r="C138" s="4" t="inlineStr">
+      <c r="C138" t="inlineStr">
         <is>
           <t>Practice With Adaptive Quizzes</t>
         </is>
       </c>
-      <c r="F138" s="5" t="inlineStr"/>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="inlineStr">
+      <c r="A139" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B139" s="3" t="inlineStr">
+      <c r="B139" t="inlineStr">
         <is>
           <t>slide2_body</t>
         </is>
       </c>
-      <c r="C139" s="4" t="inlineStr">
+      <c r="C139" t="inlineStr">
         <is>
           <t>AI generates real sentences to test you — and the more you practice, the more it targets what you're actually struggling with.</t>
         </is>
       </c>
-      <c r="F139" s="5" t="inlineStr"/>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="inlineStr">
+      <c r="A140" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B140" s="3" t="inlineStr">
+      <c r="B140" t="inlineStr">
         <is>
           <t>slide3_headline</t>
         </is>
       </c>
-      <c r="C140" s="4" t="inlineStr">
+      <c r="C140" t="inlineStr">
         <is>
           <t>Watch Your Progress</t>
         </is>
       </c>
-      <c r="F140" s="5" t="inlineStr"/>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="inlineStr">
+      <c r="A141" t="inlineStr">
         <is>
           <t>onboarding.tsx</t>
         </is>
       </c>
-      <c r="B141" s="3" t="inlineStr">
+      <c r="B141" t="inlineStr">
         <is>
           <t>slide3_body</t>
         </is>
       </c>
-      <c r="C141" s="4" t="inlineStr">
+      <c r="C141" t="inlineStr">
         <is>
           <t>See your scores improve over time, list by list.</t>
         </is>
       </c>
-      <c r="F141" s="5" t="inlineStr"/>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="inlineStr">
+      <c r="A142" t="inlineStr">
         <is>
           <t>settings.tsx</t>
         </is>
       </c>
-      <c r="B142" s="3" t="inlineStr">
+      <c r="B142" t="inlineStr">
         <is>
           <t>about_langreps_link</t>
         </is>
       </c>
-      <c r="C142" s="4" t="inlineStr">
+      <c r="C142" t="inlineStr">
         <is>
           <t>About LangReps</t>
         </is>
       </c>
-      <c r="F142" s="5" t="inlineStr">
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
         <is>
           <t>Links to /onboarding to replay it manually</t>
         </is>
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="inlineStr">
+      <c r="A143" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B143" s="3" t="inlineStr">
+      <c r="B143" t="inlineStr">
         <is>
           <t>sort_by_label</t>
         </is>
       </c>
-      <c r="C143" s="4" t="inlineStr">
+      <c r="C143" t="inlineStr">
         <is>
           <t>Sort by</t>
         </is>
       </c>
-      <c r="F143" s="5" t="inlineStr"/>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="inlineStr">
+      <c r="A144" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B144" s="3" t="inlineStr">
+      <c r="B144" t="inlineStr">
         <is>
           <t>sort_by_date</t>
         </is>
       </c>
-      <c r="C144" s="4" t="inlineStr">
+      <c r="C144" t="inlineStr">
         <is>
           <t>Last Uploaded</t>
         </is>
       </c>
-      <c r="F144" s="5" t="inlineStr"/>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr"/>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="inlineStr">
+      <c r="A145" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B145" t="inlineStr">
         <is>
           <t>sort_by_name</t>
         </is>
       </c>
-      <c r="C145" s="4" t="inlineStr">
+      <c r="C145" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="F145" s="5" t="inlineStr"/>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="inlineStr">
+      <c r="A146" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B146" s="3" t="inlineStr">
+      <c r="B146" t="inlineStr">
         <is>
           <t>last_uploaded_template</t>
         </is>
       </c>
-      <c r="C146" s="4" t="inlineStr">
+      <c r="C146" t="inlineStr">
         <is>
           <t>Last uploaded: {date}</t>
         </is>
       </c>
-      <c r="F146" s="5" t="inlineStr">
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
         <is>
           <t>Template — date formatting via toLocaleDateString(), varies by device locale</t>
         </is>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="inlineStr">
+      <c r="A147" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B147" s="3" t="inlineStr">
+      <c r="B147" t="inlineStr">
         <is>
           <t>sample_list_name_template_v2</t>
         </is>
       </c>
-      <c r="C147" s="4" t="inlineStr">
+      <c r="C147" t="inlineStr">
         <is>
           <t>{target} Vocabulary (from {source}) / {target} Verbs (from {source})</t>
         </is>
       </c>
-      <c r="F147" s="5" t="inlineStr">
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
         <is>
           <t>Superseded template — replaces the old arrow-notation naming</t>
         </is>
       </c>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="inlineStr">
+      <c r="A148" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B148" s="3" t="inlineStr">
+      <c r="B148" t="inlineStr">
         <is>
           <t>sample_list_card_title</t>
         </is>
       </c>
-      <c r="C148" s="4" t="inlineStr">
+      <c r="C148" t="inlineStr">
         <is>
           <t>Vocab {count} / Verb {count}</t>
         </is>
       </c>
-      <c r="F148" s="5" t="inlineStr">
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
         <is>
           <t>Sample-list catalog card title, replaces the old full name display</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="A149" t="inlineStr">
         <is>
           <t>my-lists.tsx</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B149" t="inlineStr">
         <is>
           <t>sample_list_card_flags</t>
         </is>
       </c>
-      <c r="C149" s="4" t="inlineStr">
+      <c r="C149" t="inlineStr">
         <is>
           <t>{flag} -&gt; {flag}</t>
         </is>
       </c>
-      <c r="F149" s="5" t="inlineStr">
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
         <is>
           <t>Flag emoji pair instead of spelled-out language names — sidesteps capitalization inconsistency entirely</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+      <c r="A150" t="inlineStr">
         <is>
           <t>index.tsx</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B150" t="inlineStr">
         <is>
           <t>signup_incentive_hint</t>
         </is>
       </c>
-      <c r="C150" s="4" t="inlineStr">
+      <c r="C150" t="inlineStr">
         <is>
           <t>Sign up to save your lists and track your progress over time</t>
         </is>
       </c>
-      <c r="F150" s="5" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Inventory of every hardcoded, user-facing string in the LangReps app (frontend UI chrome only — not vocab/quiz content, which is already language-flexible).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Key column</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>A proposed snake_case translation key for src/lib/translations/{en,es,fr}.ts (see project_langreps_localization memory note for the planned i18n architecture).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Templates</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Strings with {placeholders} are template strings — translate the surrounding text, keep the placeholder names as-is.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Spanish / French columns</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Left blank for translation — fill in when the i18n pass begins.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Backend error text</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Some error messages shown via e.message originate from the FastAPI backend (HTTPException details), not the frontend. These need either their own backend-side translation, or the frontend should map known error patterns to translated strings instead of showing raw backend text.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Not included</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Generated content (quiz questions, vocab list names, user emails) — these are inherently already in whatever language the user is studying or typed, not part of the app's UI chrome.</t>
-        </is>
-      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>default_level_title</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Default Level</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>New section title for Settings redesign (bold title + description layout)</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>auto_delete_title</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Auto-Delete Old Quizzes</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>New section title</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>auto_delete_desc</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Completed quizzes are removed after 30 days</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Description moved under the bold title</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>adaptive_quizzes_title</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Adaptive Quizzes</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>New section title</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>adaptive_quizzes_desc</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Get feedback on patterns you struggle with, and an option to target them</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr"/>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Description moved under the bold title</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>require_accents_title</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Require Accents</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>New toggle</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>require_accents_desc</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Off accepts "cafe" for "café"</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Off by default — grading strips accents; app is a reinforcement tool, not a strict teaching tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>your_lists_section_title</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Your Lists</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>New section title alongside bulk-select controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>bulk_select_toggle</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Select / Cancel</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Toggles bulk-select mode (shared pattern, My Lists and My Quizzes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>bulk_select_all</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Select All / Deselect All</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Shared pattern</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> My Lists and My Quizzes</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>bulk_delete_selected_template</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Delete Selected ({count})</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Shared pattern</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> My Lists and My Quizzes</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>bulk_deleting</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Deleting…</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Shared pattern</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> My Lists and My Quizzes</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>bulk_delete_lists_alert_title</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Delete Lists</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>bulk_delete_lists_alert_message_template</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Delete {count} list(s)? This can't be undone.</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>quizzes_in_progress_count_template</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>{count} in progress</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>bulk_delete_quizzes_alert_title</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Delete Quizzes</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>bulk_delete_quizzes_alert_message_template</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Delete {count} quiz(zes)? This can't be undone.</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Keep My Lists/My Quizzes layout stable when entering select mode
Previous version hid the sort row and each row's Progress/Delete
links while selecting, and inserted a separate bulk-action bar —
too much layout shifting. Now selecting just adds a checkbox to the
left of each row (existing row content stays put) and folds Select
All / Delete / Done into the existing header row instead of adding
a new one.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -3845,14 +3845,14 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Select / Cancel</t>
+          <t>Select / Done</t>
         </is>
       </c>
       <c r="D159" t="inlineStr"/>
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Toggles bulk-select mode (shared pattern, My Lists and My Quizzes)</t>
+          <t>Toggles bulk-select mode in the header row — rows keep their normal content, just gain a checkbox (shared pattern, My Lists and My Quizzes)</t>
         </is>
       </c>
     </row>
@@ -3898,7 +3898,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Delete Selected ({count})</t>
+          <t>Delete ({count})</t>
         </is>
       </c>
       <c r="D161" t="inlineStr"/>

</xml_diff>

<commit_message>
Add sort-by and last-updated display to My Quizzes
Mirrors My Lists: sort in-progress quizzes by Last Updated (default)
or Name (by the underlying list's name), and show each row's last
active timestamp. Uses the already-returned last_active_at field
from GET /quiz-sessions (verified against the live API — no backend
change needed).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G167"/>
+  <dimension ref="A1:G169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4043,6 +4043,54 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr"/>
     </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>sort_by_last_updated</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>New sort option — mirrors My Lists' "Last Uploaded" pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>last_updated_template</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Last updated: {date}</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr"/>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Template — date formatting via toLocaleDateString(), varies by device locale</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Show Vocab/Verb badge on My Quizzes rows
Uses list_type, already returned by GET /lists (verified: select("*")
on vocab_lists) — no backend change needed.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G169"/>
+  <dimension ref="A1:G171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4091,6 +4091,54 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>quiz_type_badge_vocab</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Vocab</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr"/>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Small badge next to the quiz row title, shows the underlying list's list_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>quiz_type_badge_verb</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Verb</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Small badge next to the quiz row title</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Always show feedback on Quiz Complete
Previously Quiz Complete showed only a bare score, and the AI pattern
insight only ever appeared pre-quiz (gated behind enough missed-word
history). Now Quiz Complete always shows a message: the AI insight
when there's enough history for a real pattern, otherwise a plain
score-based canned message (never blank).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G171"/>
+  <dimension ref="A1:G175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4139,6 +4139,102 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>quiz-complete.tsx</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>canned_feedback_perfect</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Perfect score! This list is looking solid.</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Shown when there's not yet enough history for an AI pattern insight</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>quiz-complete.tsx</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>canned_feedback_great</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Great work — you know this list well.</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr"/>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>80-99% correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>quiz-complete.tsx</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>canned_feedback_keep_going</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Keep at it — repetition is what makes this stick.</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr"/>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>50-79% correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>quiz-complete.tsx</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>canned_feedback_tough</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>This one's tough. A few more passes and it'll click.</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr"/>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Below 50% correct</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rewrite canned Quiz Complete feedback as substantive guidance
Replaces the one-line canned messages with paragraph-length feedback
that names what the score means and suggests a concrete next step
(raise CEFR level, retry the same list, lower the level, etc.),
matching the quality bar of the AI-generated insight it falls back
for.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -4147,19 +4147,19 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>canned_feedback_perfect</t>
+          <t>canned_feedback_mastery</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Perfect score! This list is looking solid.</t>
+          <t>You show mastery of the material and a good understanding of the concepts. You recall these words well and have successfully added them to your vocabulary. Keep up the good work — we suggest upping the CEFR level or training on a new list.</t>
         </is>
       </c>
       <c r="D172" t="inlineStr"/>
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
-          <t>Shown when there's not yet enough history for an AI pattern insight</t>
+          <t>Shown when there's not yet enough history for an AI pattern insight. 90%+ correct</t>
         </is>
       </c>
     </row>
@@ -4171,19 +4171,19 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>canned_feedback_great</t>
+          <t>canned_feedback_solid</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Great work — you know this list well.</t>
+          <t>You have a solid grasp of this list — most of these words are sticking. A few are still slipping through, so one more pass at this level should lock them in before you move up or take on a new list.</t>
         </is>
       </c>
       <c r="D173" t="inlineStr"/>
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>80-99% correct</t>
+          <t>70-89% correct</t>
         </is>
       </c>
     </row>
@@ -4195,19 +4195,19 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>canned_feedback_keep_going</t>
+          <t>canned_feedback_building</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Keep at it — repetition is what makes this stick.</t>
+          <t>You're recognizing some of these words, but a good chunk aren't sticking yet. That's normal at this stage — stick with this list at the same level for now rather than adding new words.</t>
         </is>
       </c>
       <c r="D174" t="inlineStr"/>
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>50-79% correct</t>
+          <t>40-69% correct</t>
         </is>
       </c>
     </row>
@@ -4219,19 +4219,19 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>canned_feedback_tough</t>
+          <t>canned_feedback_struggling</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>This one's tough. A few more passes and it'll click.</t>
+          <t>This list is still tripping you up more than not — that's useful information, not a setback. Try lowering the CEFR level or running a shorter, more focused quiz on just this list before moving on.</t>
         </is>
       </c>
       <c r="D175" t="inlineStr"/>
       <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Below 50% correct</t>
+          <t>Below 40% correct</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add info icon explaining CEFR levels
Small ⓘ next to the Level label on CefrLevelPicker (used on Generate
Quiz and Settings) opens a plain-language summary of what A1-C2
actually mean, so a first-time user isn't left guessing.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G175"/>
+  <dimension ref="A1:G182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4235,6 +4235,150 @@
         </is>
       </c>
     </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>cefr-level-picker.tsx</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>cefr_info_alert_title</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>CEFR Levels</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Alert title triggered by new info icon next to the Level label</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>cefr-level-picker.tsx</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>cefr_a1_explanation</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Breakthrough — basic words and phrases for everyday needs.</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr"/>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>cefr-level-picker.tsx</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>cefr_a2_explanation</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Waystage — simple sentences about familiar topics like family and shopping.</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr"/>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>cefr-level-picker.tsx</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>cefr_b1_explanation</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Threshold — comfortable with everyday situations, travel, and routine topics.</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr"/>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>cefr-level-picker.tsx</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>cefr_b2_explanation</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Vantage — can discuss general and some abstract topics with varied vocabulary.</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>cefr-level-picker.tsx</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>cefr_c1_explanation</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Advanced — fluent, spontaneous use for social, academic, or work purposes.</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr"/>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>cefr-level-picker.tsx</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>cefr_c2_explanation</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Mastery — near-native fluency with precise, nuanced expression.</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr"/>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename Require Accents toggle to Require Diacritics
Label only — storage key, function names, and behavior unchanged.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -3773,14 +3773,14 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Require Accents</t>
+          <t>Require Diacritics</t>
         </is>
       </c>
       <c r="D156" t="inlineStr"/>
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
-          <t>New toggle</t>
+          <t>New toggle — renamed from "Require Accents"</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add branded Welcome screen before onboarding
New users previously landed straight on the onboarding slides with
no branding at all. Adds src/app/welcome.tsx (LangReps title,
tagline, Get Started button, "© 2026 MarApps Development" pinned in
the bottom-right corner) as the actual first screen; Home now routes
first-time users there instead of straight into onboarding.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G182"/>
+  <dimension ref="A1:G186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4379,6 +4379,99 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr"/>
     </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>welcome.tsx</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>welcome_title</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>LangReps</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>New branded first screen shown before onboarding slides — proper name</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> may stay untranslated</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>welcome.tsx</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>welcome_tagline</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Language reps that stick.</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>welcome.tsx</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>get_started</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Get Started</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr"/>
+      <c r="F185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>welcome.tsx</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>copyright</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>© 2026 MarApps Development</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Pinned bottom-right corner</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Replace first-time welcome screen with an every-launch animated splash
Supersedes the previous welcome.tsx (shown once, before onboarding)
with src/components/app-splash.tsx: a fade+scale-in LangReps splash
shown on every app launch via a new AppGate in _layout.tsx, gated on
auth's isLoading plus a minimum visible duration (1100ms) so it
never flashes by unseen on a fast restore. Onboarding's own
first-time gating (Home -> /onboarding) is unchanged.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G186"/>
+  <dimension ref="A1:G185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4382,12 +4382,12 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>welcome.tsx</t>
+          <t>app-splash.tsx</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>welcome_title</t>
+          <t>splash_title</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4399,24 +4399,19 @@
       <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
         <is>
-          <t>New branded first screen shown before onboarding slides — proper name</t>
-        </is>
-      </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> may stay untranslated</t>
+          <t>Animated splash shown on every app launch (not a navigable screen) — proper name, may stay untranslated</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>welcome.tsx</t>
+          <t>app-splash.tsx</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>welcome_tagline</t>
+          <t>splash_tagline</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4431,42 +4426,22 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>welcome.tsx</t>
+          <t>app-splash.tsx</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>get_started</t>
+          <t>splash_copyright</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Get Started</t>
+          <t>© 2026 MarApps Development</t>
         </is>
       </c>
       <c r="D185" t="inlineStr"/>
       <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr"/>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>welcome.tsx</t>
-        </is>
-      </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>copyright</t>
-        </is>
-      </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>© 2026 MarApps Development</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr"/>
-      <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr">
+      <c r="F185" t="inlineStr">
         <is>
           <t>Pinned bottom-right corner</t>
         </is>

</xml_diff>

<commit_message>
Add full quiz results screen with color-coded correct/incorrect rows
New src/app/quiz-results.tsx: scrollable table of every question,
your answer, and the correct answer, fetched from the new
GET /quiz-sessions/{id}/attempts endpoint — green left-border for
correct rows, red for incorrect (correct answer only shown when
wrong). Linked from Quiz Complete via "See Full Results", shown only
for saved-list quizzes (a session must exist).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4447,6 +4447,158 @@
         </is>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>quiz-complete.tsx</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>see_full_results</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>See Full Results</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Link to the new quiz-results.tsx screen, only shown for saved-list quizzes (a session exists)</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>quiz-results.tsx</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>full_results_title</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Full Results</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr"/>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>quiz-results.tsx</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>no_recorded_answers</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>No recorded answers for this quiz.</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr"/>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>quiz-results.tsx</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>your_answer_label</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Your answer:</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr"/>
+      <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>quiz-results.tsx</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>correct_answer_label</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Correct answer:</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr"/>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Shown only for incorrect rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>quiz-results.tsx</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>blank_answer_fallback</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>(blank)</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr"/>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Shown when a skipped/empty answer was recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>quiz-results.tsx</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>error_loading_results</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Something went wrong loading results.</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr"/>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix tiny Dropdown value text, add List Type info icon
Dropdown's selected-value Text had no explicit style at all, so it
rendered at a tiny system default regardless of surrounding sizing —
now 16px/600 weight, fixing this for every Dropdown usage app-wide,
not just List type. Also added a "List type" label style (was using
shared.hint, too small/faint for a field label) and an info icon
explaining what Vocab vs Verb actually changes about a quiz.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G192"/>
+  <dimension ref="A1:G195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4599,6 +4599,70 @@
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr"/>
     </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>list_type_info_alert_title</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>List Types</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr"/>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>New info icon next to the List type label</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>list_type_info_vocab</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Vocab — plain word pairs (nouns, adjectives, etc.), tested as-is.</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr"/>
+      <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>list_type_info_verb</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Verb — infinitives get conjugated in context on Generate Quiz, so you're tested on actual verb forms (e.g. "habla") instead of just recalling the infinitive ("hablar").</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr"/>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add persistent label above Save List name field
Was placeholder-only ("List name"), which disappears once you start
typing and was apparently not a strong enough cue that the field is
for the list's name. Now has a real label above it that stays visible
while typing, plus a concrete example as the placeholder instead.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G195"/>
+  <dimension ref="A1:G198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4663,6 +4663,83 @@
       <c r="E195" t="inlineStr"/>
       <c r="F195" t="inlineStr"/>
     </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>save_label_new</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Name this list to save it</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr"/>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>New persistent label above the name field, was placeholder-only before</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>save_label_update</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>List name (saving updates it)</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr"/>
+      <c r="E197" t="inlineStr"/>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Moved from placeholder to a persistent label above the field</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>save_input_placeholder</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>e.g. Spanish Verbs</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr"/>
+      <c r="E198" t="inlineStr"/>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>New example placeholder</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> replaces the old "List name" placeholder now that a persistent label exists</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert Save List label to placeholder-only
The separate label above the field felt too busy — back to a single
placeholder inside the input, just with clearer wording than the
original bare "List name".
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G198"/>
+  <dimension ref="A1:G197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>save_label_new</t>
+          <t>save_input_placeholder_new</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -4683,7 +4683,7 @@
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
-          <t>New persistent label above the name field, was placeholder-only before</t>
+          <t>Placeholder text (reverted from a separate label above the field — felt too busy)</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>save_label_update</t>
+          <t>save_input_placeholder_update</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4707,36 +4707,7 @@
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Moved from placeholder to a persistent label above the field</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>pairs-review.tsx</t>
-        </is>
-      </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>save_input_placeholder</t>
-        </is>
-      </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>e.g. Spanish Verbs</t>
-        </is>
-      </c>
-      <c r="D198" t="inlineStr"/>
-      <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr">
-        <is>
-          <t>New example placeholder</t>
-        </is>
-      </c>
-      <c r="G198" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> replaces the old "List name" placeholder now that a persistent label exists</t>
+          <t>Placeholder shown once the list is already saved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix invisible placeholder text app-wide, shorten Save List placeholder
Root cause of "I don't see the placeholder": no TextInput anywhere in
the app set placeholderTextColor, so all of them fell back to iOS's
default light gray — poor contrast against this app's cream
background, effectively invisible. Added colors.placeholder and
applied it to every TextInput (Save List, Add Words, Paste, Login,
Quiz answer). Also shortened Save List's placeholder text since the
longer version didn't fit next to the Save button.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G197"/>
+  <dimension ref="A1:G198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4676,14 +4676,14 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Name this list to save it</t>
+          <t>Name this list</t>
         </is>
       </c>
       <c r="D196" t="inlineStr"/>
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Placeholder text (reverted from a separate label above the field — felt too busy)</t>
+          <t>Placeholder text — shortened from "Name this list to save it", didn't fit alongside the Save button</t>
         </is>
       </c>
     </row>
@@ -4700,14 +4700,34 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>List name (saving updates it)</t>
+          <t>List name (updates it)</t>
         </is>
       </c>
       <c r="D197" t="inlineStr"/>
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Placeholder shown once the list is already saved</t>
+          <t>Placeholder shown once the list is already saved — shortened to fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>constants/styles.ts</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>placeholder_color_note</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr"/>
+      <c r="D198" t="inlineStr"/>
+      <c r="E198" t="inlineStr"/>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Not a UI string — new colors.placeholder token (#8C7F63) applied via placeholderTextColor to every TextInput app-wide; RN's default placeholder gray had poor contrast on the parchment background and was nearly invisible</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add saved-list editing: Edit link on My Lists, per-word remove
Previously a saved list could only be quizzed or deleted, never
edited. My Lists rows gain an "Edit" action that loads the list into
Add Words (reusing save-by-name's existing update-in-place behavior)
instead of always jumping to Generate Quiz. PairsReview's word list
also gains a per-row "✕" remove button — previously the only removal
options were Undo last (most recent only) or Clear list (everything).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G198"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4731,6 +4731,54 @@
         </is>
       </c>
     </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>edit_list_link</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr"/>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>New row action — loads the list into Add Words for editing instead of only Generate Quiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>remove_word_icon</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>✕</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>New per-word remove button in the word list, was append/undo-last/clear-all only before</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Wire translate-monolingual-list into Upload File and Paste
New TranslateSkippedLines component shows under a parse's "couldn't
parse N lines" message: pick a target language, hit Translate, and
those leftover single-word lines (e.g. a textbook vocab list with no
translations) get turned into real pairs via the new
/translate-word-list endpoint. Detected source language and the
chosen target both get applied to the list's language picker.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4779,6 +4779,119 @@
         </is>
       </c>
     </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>translate-skipped-lines.tsx</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>translate_prompt_template</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>{n} line(s) looked like single word(s)</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> not pairs — translate into:</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>New — shown under a parse's "couldn't parse N lines" message on Upload File and Paste</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>translate-skipped-lines.tsx</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>translate_button</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Translate</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr"/>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>translate-skipped-lines.tsx</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>translating_ellipsis</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Translating…</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr"/>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>translate-skipped-lines.tsx</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>error_translating</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Something went wrong translating those words.</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr"/>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>slide1_body_updated</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Type words, paste a list, or upload a file — AI reads it for you. Or jump right in with a few ready-made sample lists in My Lists.</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr"/>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>Updated — removed "or snap a photo" since Upload Photo was tabled</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Show saved list's name prominently once labeled and saved
PairsReview now displays the list's own name at the top (styled like
Generate Quiz's heading) once savedListId is set — previously the
only indication you were working on a saved list was the small
"(updates it)" placeholder hint on the name field, easy to miss
especially on the new Edit List flow.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G205"/>
+  <dimension ref="A1:G206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4892,6 +4892,26 @@
         </is>
       </c>
     </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>saved_list_heading</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr"/>
+      <c r="D206" t="inlineStr"/>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>Not new text — shows the list's own saved name prominently at the top of PairsReview once saved (Edit flow especially), styled like Generate Quiz's list-name heading</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Separate renaming a saved list from saving its pairs
Previously the only save path was save_list()'s upsert-by-name, so
changing the name field and hitting Save would silently create a
duplicate list rather than renaming the existing one. Now:
- A new list (no savedListId yet) still needs a name to save for the
  first time — unchanged, still uses the name-based create path.
- An already-saved list shows its name as a heading with a separate
  "Rename" action (PATCH /lists/{id}, name only), and a "Save
  Changes" button that updates pairs by id (PUT /lists/{id}, no name
  field at all) — editing words can no longer risk creating a
  duplicate under a different name.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G206"/>
+  <dimension ref="A1:G211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4912,6 +4912,122 @@
         </is>
       </c>
     </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>rename_link</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Rename</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr"/>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>New — separates renaming an already-saved list from saving its pairs</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>rename_save_button</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Save</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr"/>
+      <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>Inline rename confirm button</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>rename_cancel_button</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Cancel</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr"/>
+      <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Inline rename cancel button</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>error_renaming</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Something went wrong renaming.</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr"/>
+      <c r="E210" t="inlineStr"/>
+      <c r="F210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>save_changes_button</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Save Changes</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr"/>
+      <c r="E211" t="inlineStr"/>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>Replaces "Save List"+name field once a list is already saved — updates pairs by id, no name field</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Move Undo/Clear below Add to list, lock List type after first save
- Undo last/Clear list now render after the screen-specific "add
  more" UI (children) instead of before it, closer to the word list
  they affect.
- List type dropdown is now disabled once a list is saved (label
  shows "(locked)", info alert explains why: quiz history is tied to
  how a word is tested, so switching types on an existing list would
  make past results inconsistent).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G211"/>
+  <dimension ref="A1:G213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5028,6 +5028,54 @@
         </is>
       </c>
     </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>list_type_locked_label</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>List type (locked)</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr"/>
+      <c r="E212" t="inlineStr"/>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>Appended to the label once a list is saved — type can't change after first save</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>list_type_locked_explanation</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Can't be changed after a list is saved — quiz history is tied to how a word is tested, so switching types on an existing list would make its past results inconsistent. Save a new list instead if you need the other type.</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>Appended to the existing List Types info alert once locked</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Past Quizzes section to My Quizzes
Previously only in-progress sessions were shown. New section lists
completed quizzes (name, score, date) fetched from the new
GET /quiz-sessions/completed — tapping one opens the existing Full
Results screen (reuses quiz-results.tsx, since attempts are recorded
regardless of completion status), with its own delete action.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G213"/>
+  <dimension ref="A1:G217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5076,6 +5076,103 @@
         </is>
       </c>
     </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>past_quizzes_section_title</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Past Quizzes</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr"/>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>New section showing completed quiz history</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> fetched from GET /quiz-sessions/completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>no_completed_quizzes</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>No completed quizzes yet.</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>past_quiz_score_template</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>{correct}/{total} correct ({pct}%)</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr"/>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>Template</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>deleted_list_fallback</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Deleted list</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr"/>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>Shown when a past quiz's list no longer exists</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Confirm before discarding 3+ unsaved manually-added words
BackButton gains an optional confirmLeave prop — Add Words passes
one that fires when there's no savedListId yet (a fresh, never-saved
list) and 3+ pairs have been added, showing an Alert before actually
navigating away. Other screens' BackButton usage is unaffected
(confirmLeave omitted = navigates straight through, same as before).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G217"/>
+  <dimension ref="A1:G220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5173,6 +5173,74 @@
         </is>
       </c>
     </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>back-button.tsx</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>discard_unsaved_alert_title</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Discard unsaved words?</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr"/>
+      <c r="E218" t="inlineStr"/>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>New — shown when backing out of Add Words with 3+ unsaved words</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>back-button.tsx</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>discard_unsaved_alert_message</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>You've added words that haven't been saved yet. Leaving now will lose them.</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>back-button.tsx</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>leave_without_saving</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Leave Without Saving</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>Destructive confirm action</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Simplify language labels to From/To
"I already know"/"I'm learning" and their later "Known"/"Learning"
revision both had the same problem: awkward or ungrammatical once
translated (needs gender agreement, reads as an incomplete gerund).
"From"/"To" is the standard translation-app convention and translates
cleanly everywhere. Also dropped the now-redundant "(known)"/
"(learning)" qualifiers on Add Words' input placeholders, since the
picker directly above already establishes direction — just "Word in
{language}" for both.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -1264,7 +1264,12 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Superseded by source_word_placeholder_dynamic — was static, replaced with actual language name + known/learning framing</t>
+          <t>Superseded by source_word_placeholder_dynamic — was static</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> replaced with actual language name</t>
         </is>
       </c>
     </row>
@@ -3692,25 +3697,29 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>i_already_know</t>
+          <t>from_label</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>I already know</t>
+          <t>From</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Ya sé</t>
+          <t>Desde</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Je connais déjà</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr"/>
+          <t>Depuis</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Replaces "I already know" — short label translates cleanly, standard in translation-app pickers (Google Translate, Duolingo-style)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3720,25 +3729,29 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>i_am_learning</t>
+          <t>to_label</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>I'm learning</t>
+          <t>To</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Estoy aprendiendo</t>
+          <t>Hacia</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>J'apprends</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr"/>
+          <t>Vers</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Replaces "I'm learning" — same reasoning</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6967,22 +6980,22 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Word in {language} (known)</t>
+          <t>Word in {language}</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Palabra en {language} (conocido)</t>
+          <t>Palabra en {language}</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Mot en {language} (connu)</t>
+          <t>Mot en {language}</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Replaces static "Source word" placeholder — shows actual selected language + known/learning framing instead of source/target jargon</t>
+          <t>Simplified — dropped "(known)" qualifier, the From/To picker above already establishes direction</t>
         </is>
       </c>
     </row>
@@ -6999,22 +7012,22 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Word in {language} (learning)</t>
+          <t>Word in {language}</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Palabra en {language} (aprendiendo)</t>
+          <t>Palabra en {language}</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Mot en {language} (en apprentissage)</t>
+          <t>Mot en {language}</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Replaces static "Target word" placeholder</t>
+          <t>Simplified — dropped "(learning)" qualifier, same reasoning</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish Dropdown affordance, Generate Quiz UX, and drop manual app-language setting
- Dropdown gains a visible chevron so every picker in the app (tense,
  language, sort, list type) reads as tappable instead of a static field.
- Generate Quiz: haptic feedback on generating a quiz (success/error too,
  matching the existing quiz-flow pattern), and fixed the back arrow
  sitting too low (the screen centered its whole content as one group,
  including the arrow — now the arrow is pinned to the top like every
  other screen while the rest of the content still centers itself).
- Removed the manual App Language setting entirely — with no UI ever
  calling it beyond that one picker, the persisted-override machinery in
  i18n.tsx was dead weight; the app now simply follows the device's
  language at launch, same default behavior as before minus the override.
- Restored the "Require Diacritics" explanation text that was dropped
  when accent-leniency became a per-language-pair setting.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -8523,32 +8523,32 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>settings.tsx</t>
+          <t>pairs-review.tsx</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>app_language_title</t>
+          <t>list_type_label</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>App Language</t>
+          <t>List type</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>Idioma de la app</t>
+          <t>Tipo de lista</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>Langue de l'application</t>
+          <t>Type de liste</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>New — the UI locale picker itself, part of building the actual i18n layer</t>
+          <t>New — plain unlocked label; list_type_locked_label is the separate (locked) variant</t>
         </is>
       </c>
     </row>
@@ -8560,32 +8560,32 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>pairs-review.tsx</t>
+          <t>my-lists.tsx</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>list_type_label</t>
+          <t>select_label</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>List type</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Tipo de lista</t>
+          <t>Seleccionar</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Type de liste</t>
+          <t>Sélectionner</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>New — plain unlocked label; list_type_locked_label is the separate (locked) variant</t>
+          <t>Split from the old combined "Select / Done" doc row — separate key needed for actual t() usage. Shared pattern, My Lists and My Quizzes</t>
         </is>
       </c>
     </row>
@@ -8602,27 +8602,27 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>select_label</t>
+          <t>done_label</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Select</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Seleccionar</t>
+          <t>Listo</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Sélectionner</t>
+          <t>Terminé</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Split from the old combined "Select / Done" doc row — separate key needed for actual t() usage. Shared pattern, My Lists and My Quizzes</t>
+          <t>Split from "Select / Done". Shared pattern, My Lists and My Quizzes</t>
         </is>
       </c>
     </row>
@@ -8639,27 +8639,27 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>done_label</t>
+          <t>select_all_label</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Select All</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Listo</t>
+          <t>Seleccionar todo</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Terminé</t>
+          <t>Tout sélectionner</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
-          <t>Split from "Select / Done". Shared pattern, My Lists and My Quizzes</t>
+          <t>Split from "Select All / Deselect All". Shared pattern, My Lists and My Quizzes</t>
         </is>
       </c>
     </row>
@@ -8676,22 +8676,22 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>select_all_label</t>
+          <t>deselect_all_label</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Select All</t>
+          <t>Deselect All</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Seleccionar todo</t>
+          <t>Deseleccionar todo</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Tout sélectionner</t>
+          <t>Tout désélectionner</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -8713,27 +8713,27 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>deselect_all_label</t>
+          <t>error_deleting_lists_bulk</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Deselect All</t>
+          <t>Something went wrong deleting those lists.</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Deseleccionar todo</t>
+          <t>Algo salió mal al eliminar esas listas.</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Tout désélectionner</t>
+          <t>Une erreur s'est produite lors de la suppression de ces listes.</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>Split from "Select All / Deselect All". Shared pattern, My Lists and My Quizzes</t>
+          <t>Plural — bulk-delete error, distinct from error_deleting_list (singular)</t>
         </is>
       </c>
     </row>
@@ -8745,32 +8745,32 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>my-lists.tsx</t>
+          <t>my-quizzes.tsx</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>error_deleting_lists_bulk</t>
+          <t>error_deleting_quizzes_bulk</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Something went wrong deleting those lists.</t>
+          <t>Something went wrong deleting those quizzes.</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>Algo salió mal al eliminar esas listas.</t>
+          <t>Algo salió mal al eliminar esos cuestionarios.</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Une erreur s'est produite lors de la suppression de ces listes.</t>
+          <t>Une erreur s'est produite lors de la suppression de ces quiz.</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
-          <t>Plural — bulk-delete error, distinct from error_deleting_list (singular)</t>
+          <t>Plural — bulk-delete error, distinct from error_deleting_quiz (singular)</t>
         </is>
       </c>
     </row>
@@ -8782,32 +8782,32 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>my-quizzes.tsx</t>
+          <t>my-lists.tsx</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>error_deleting_quizzes_bulk</t>
+          <t>loading_ellipsis</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Something went wrong deleting those quizzes.</t>
+          <t>Loading…</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Algo salió mal al eliminar esos cuestionarios.</t>
+          <t>Cargando…</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Une erreur s'est produite lors de la suppression de ces quiz.</t>
+          <t>Chargement…</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>Plural — bulk-delete error, distinct from error_deleting_quiz (singular)</t>
+          <t>Reused wherever a screen shows a generic loading state</t>
         </is>
       </c>
     </row>
@@ -8819,34 +8819,30 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>my-lists.tsx</t>
+          <t>login.tsx</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>loading_ellipsis</t>
+          <t>forgot_password_link</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Loading…</t>
+          <t>Forgot password?</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Cargando…</t>
+          <t>¿Olvidaste tu contraseña?</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Chargement…</t>
-        </is>
-      </c>
-      <c r="G243" t="inlineStr">
-        <is>
-          <t>Reused wherever a screen shows a generic loading state</t>
-        </is>
-      </c>
+          <t>Mot de passe oublié ?</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -8856,27 +8852,27 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>login.tsx</t>
+          <t>forgot-password.tsx</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>forgot_password_link</t>
+          <t>forgot_password_title</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Forgot password?</t>
+          <t>Forgot Password</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>¿Olvidaste tu contraseña?</t>
+          <t>Contraseña olvidada</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Mot de passe oublié ?</t>
+          <t>Mot de passe oublié</t>
         </is>
       </c>
       <c r="G244" t="inlineStr"/>
@@ -8894,25 +8890,29 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>forgot_password_title</t>
+          <t>forgot_password_sent_message</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Forgot Password</t>
+          <t>If an account exists for that email, we've sent a link to reset your password. Check your inbox.</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Contraseña olvidada</t>
+          <t>Si existe una cuenta con ese correo, te hemos enviado un enlace para restablecer tu contraseña. Revisa tu bandeja de entrada.</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>Mot de passe oublié</t>
-        </is>
-      </c>
-      <c r="G245" t="inlineStr"/>
+          <t>Si un compte existe pour cette adresse e-mail, nous t'avons envoyé un lien pour réinitialiser ton mot de passe. Vérifie ta boîte de réception.</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Deliberately non-revealing — matches backend's response regardless of whether the email has an account</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -8927,29 +8927,25 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>forgot_password_sent_message</t>
+          <t>forgot_password_instructions</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>If an account exists for that email, we've sent a link to reset your password. Check your inbox.</t>
+          <t>Enter your email and we'll send you a link to reset your password.</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Si existe una cuenta con ese correo, te hemos enviado un enlace para restablecer tu contraseña. Revisa tu bandeja de entrada.</t>
+          <t>Introduce tu correo y te enviaremos un enlace para restablecer tu contraseña.</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Si un compte existe pour cette adresse e-mail, nous t'avons envoyé un lien pour réinitialiser ton mot de passe. Vérifie ta boîte de réception.</t>
-        </is>
-      </c>
-      <c r="G246" t="inlineStr">
-        <is>
-          <t>Deliberately non-revealing — matches backend's response regardless of whether the email has an account</t>
-        </is>
-      </c>
+          <t>Entre ton e-mail et nous t'enverrons un lien pour réinitialiser ton mot de passe.</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -8964,22 +8960,22 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>forgot_password_instructions</t>
+          <t>sending_ellipsis</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Enter your email and we'll send you a link to reset your password.</t>
+          <t>Sending…</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Introduce tu correo y te enviaremos un enlace para restablecer tu contraseña.</t>
+          <t>Enviando…</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Entre ton e-mail et nous t'enverrons un lien pour réinitialiser ton mot de passe.</t>
+          <t>Envoi en cours…</t>
         </is>
       </c>
       <c r="G247" t="inlineStr"/>
@@ -8997,22 +8993,22 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>sending_ellipsis</t>
+          <t>send_reset_link</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Sending…</t>
+          <t>Send Reset Link</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Enviando…</t>
+          <t>Enviar enlace de restablecimiento</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Envoi en cours…</t>
+          <t>Envoyer le lien de réinitialisation</t>
         </is>
       </c>
       <c r="G248" t="inlineStr"/>
@@ -9025,27 +9021,27 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>forgot-password.tsx</t>
+          <t>reset-password.tsx</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>send_reset_link</t>
+          <t>reset_password_title</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Send Reset Link</t>
+          <t>Reset Password</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Enviar enlace de restablecimiento</t>
+          <t>Restablecer contraseña</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Envoyer le lien de réinitialisation</t>
+          <t>Réinitialiser le mot de passe</t>
         </is>
       </c>
       <c r="G249" t="inlineStr"/>
@@ -9063,22 +9059,22 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>reset_password_title</t>
+          <t>reset_link_invalid_message</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Reset Password</t>
+          <t>This link looks invalid or expired. Request a new reset link from the login screen.</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Restablecer contraseña</t>
+          <t>Este enlace parece no válido o ha caducado. Solicita un nuevo enlace desde la pantalla de inicio de sesión.</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Réinitialiser le mot de passe</t>
+          <t>Ce lien semble invalide ou expiré. Demande un nouveau lien depuis l'écran de connexion.</t>
         </is>
       </c>
       <c r="G250" t="inlineStr"/>
@@ -9096,22 +9092,22 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>reset_link_invalid_message</t>
+          <t>set_new_password_title</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>This link looks invalid or expired. Request a new reset link from the login screen.</t>
+          <t>Set a New Password</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Este enlace parece no válido o ha caducado. Solicita un nuevo enlace desde la pantalla de inicio de sesión.</t>
+          <t>Establece una nueva contraseña</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Ce lien semble invalide ou expiré. Demande un nouveau lien depuis l'écran de connexion.</t>
+          <t>Définis un nouveau mot de passe</t>
         </is>
       </c>
       <c r="G251" t="inlineStr"/>
@@ -9129,22 +9125,22 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>set_new_password_title</t>
+          <t>new_password_placeholder</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Set a New Password</t>
+          <t>New password</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Establece una nueva contraseña</t>
+          <t>Nueva contraseña</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Définis un nouveau mot de passe</t>
+          <t>Nouveau mot de passe</t>
         </is>
       </c>
       <c r="G252" t="inlineStr"/>
@@ -9162,22 +9158,22 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>new_password_placeholder</t>
+          <t>save_new_password</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>New password</t>
+          <t>Save New Password</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Nueva contraseña</t>
+          <t>Guardar nueva contraseña</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Nouveau mot de passe</t>
+          <t>Enregistrer le nouveau mot de passe</t>
         </is>
       </c>
       <c r="G253" t="inlineStr"/>
@@ -9190,30 +9186,34 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>reset-password.tsx</t>
+          <t>list-details.tsx</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>save_new_password</t>
+          <t>sort_by_added_order</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Save New Password</t>
+          <t>Order Added</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Guardar nueva contraseña</t>
+          <t>Orden de añadido</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Enregistrer le nouveau mot de passe</t>
-        </is>
-      </c>
-      <c r="G254" t="inlineStr"/>
+          <t>Ordre d'ajout</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Word-list sort option — mirrors My Lists' sort-by pattern; default order (insertion order)</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -9228,29 +9228,25 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>sort_by_added_order</t>
+          <t>bulk_delete_words_alert_title</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Order Added</t>
+          <t>Delete Words</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Orden de añadido</t>
+          <t>Eliminar palabras</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Ordre d'ajout</t>
-        </is>
-      </c>
-      <c r="G255" t="inlineStr">
-        <is>
-          <t>Word-list sort option — mirrors My Lists' sort-by pattern; default order (insertion order)</t>
-        </is>
-      </c>
+          <t>Supprimer les mots</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -9265,25 +9261,29 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>bulk_delete_words_alert_title</t>
+          <t>bulk_delete_words_alert_message_template</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Delete Words</t>
+          <t>Delete {count} word(s)? This can't be undone.</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Eliminar palabras</t>
+          <t>¿Eliminar {count} palabra(s)? Esta acción no se puede deshacer.</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Supprimer les mots</t>
-        </is>
-      </c>
-      <c r="G256" t="inlineStr"/>
+          <t>Supprimer {count} mot(s) ? Cette action est irréversible.</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>Template</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -9293,32 +9293,32 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>list-details.tsx</t>
+          <t>my-lists.tsx</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>bulk_delete_words_alert_message_template</t>
+          <t>sample_category_common_words</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Delete {count} word(s)? This can't be undone.</t>
+          <t>Common Words</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>¿Eliminar {count} palabra(s)? Esta acción no se puede deshacer.</t>
+          <t>Palabras comunes</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Supprimer {count} mot(s) ? Cette action est irréversible.</t>
+          <t>Mots courants</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>Template</t>
+          <t>Sample-list category label</t>
         </is>
       </c>
     </row>
@@ -9335,22 +9335,22 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>sample_category_common_words</t>
+          <t>sample_category_common_verbs</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Common Words</t>
+          <t>Common Verbs</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Palabras comunes</t>
+          <t>Verbos comunes</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Mots courants</t>
+          <t>Verbes courants</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -9372,27 +9372,27 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>sample_category_common_verbs</t>
+          <t>sample_category_irregular_verbs</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Common Verbs</t>
+          <t>Irregular Verbs</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Verbos comunes</t>
+          <t>Verbos irregulares</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Verbes courants</t>
+          <t>Verbes irréguliers</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>Sample-list category label</t>
+          <t>Sample-list category label — new dedicated dataset, distinct from Common Verbs</t>
         </is>
       </c>
     </row>
@@ -9409,27 +9409,27 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>sample_category_irregular_verbs</t>
+          <t>sample_category_food</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Irregular Verbs</t>
+          <t>Food Words</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Verbos irregulares</t>
+          <t>Palabras de comida</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Verbes irréguliers</t>
+          <t>Mots de nourriture</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>Sample-list category label — new dedicated dataset, distinct from Common Verbs</t>
+          <t>Sample-list category label — new dedicated dataset</t>
         </is>
       </c>
     </row>
@@ -9441,34 +9441,30 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>my-lists.tsx</t>
+          <t>settings.tsx</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>sample_category_food</t>
+          <t>learning_pair_title</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Food Words</t>
+          <t>What are you learning?</t>
         </is>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Palabras de comida</t>
+          <t>¿Qué estás aprendiendo?</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Mots de nourriture</t>
-        </is>
-      </c>
-      <c r="G261" t="inlineStr">
-        <is>
-          <t>Sample-list category label — new dedicated dataset</t>
-        </is>
-      </c>
+          <t>Qu'apprends-tu ?</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -9483,25 +9479,29 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>learning_pair_title</t>
+          <t>learning_pair_hint</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>What are you learning?</t>
+          <t>Add every language you're learning — each gets its own level and starter lists.</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>¿Qué estás aprendiendo?</t>
+          <t>Añade cada idioma que estás aprendiendo — cada uno tiene su propio nivel y sus propias listas iniciales.</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Qu'apprends-tu ?</t>
-        </is>
-      </c>
-      <c r="G262" t="inlineStr"/>
+          <t>Ajoute chaque langue que tu apprends — chacune a son propre niveau et ses propres listes de départ.</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Updated for multi-language support — was singular ('your default pair'), now plural</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -9516,27 +9516,27 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>learning_pair_hint</t>
+          <t>generating_starter_lists</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Add every language you're learning — each gets its own level and starter lists.</t>
+          <t>Setting up your starter lists…</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Añade cada idioma que estás aprendiendo — cada uno tiene su propio nivel y sus propias listas iniciales.</t>
+          <t>Preparando tus listas iniciales…</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Ajoute chaque langue que tu apprends — chacune a son propre niveau et ses propres listes de départ.</t>
+          <t>Préparation de tes listes de départ…</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Updated for multi-language support — was singular ('your default pair'), now plural</t>
+          <t>Shown while the first-time PATCH /me/profile call is generating sample lists via Gemini</t>
         </is>
       </c>
     </row>
@@ -9553,29 +9553,25 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>generating_starter_lists</t>
+          <t>starter_lists_ready_message</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Setting up your starter lists…</t>
+          <t>Your starter lists are ready — check My Lists!</t>
         </is>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Preparando tus listas iniciales…</t>
+          <t>¡Tus listas iniciales ya están listas — échales un vistazo en Mis listas!</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Préparation de tes listes de départ…</t>
-        </is>
-      </c>
-      <c r="G264" t="inlineStr">
-        <is>
-          <t>Shown while the first-time PATCH /me/profile call is generating sample lists via Gemini</t>
-        </is>
-      </c>
+          <t>Tes listes de départ sont prêtes — jette un œil dans Mes listes !</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -9590,22 +9586,22 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>starter_lists_ready_message</t>
+          <t>add_language_button</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Your starter lists are ready — check My Lists!</t>
+          <t>Add Language</t>
         </is>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>¡Tus listas iniciales ya están listas — échales un vistazo en Mis listas!</t>
+          <t>Añadir idioma</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Tes listes de départ sont prêtes — jette un œil dans Mes listes !</t>
+          <t>Ajouter une langue</t>
         </is>
       </c>
       <c r="G265" t="inlineStr"/>
@@ -9623,22 +9619,22 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>add_language_button</t>
+          <t>no_languages_added</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Add Language</t>
+          <t>No languages added yet — add one below to get started.</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Añadir idioma</t>
+          <t>Aún no has añadido ningún idioma — añade uno abajo para empezar.</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Ajouter une langue</t>
+          <t>Tu n'as encore ajouté aucune langue — ajoutes-en une ci-dessous pour commencer.</t>
         </is>
       </c>
       <c r="G266" t="inlineStr"/>
@@ -9656,25 +9652,29 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>no_languages_added</t>
+          <t>remove_language_confirm_title</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>No languages added yet — add one below to get started.</t>
+          <t>Remove language?</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Aún no has añadido ningún idioma — añade uno abajo para empezar.</t>
+          <t>¿Eliminar idioma?</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Tu n'as encore ajouté aucune langue — ajoutes-en une ci-dessous pour commencer.</t>
-        </is>
-      </c>
-      <c r="G267" t="inlineStr"/>
+          <t>Supprimer la langue ?</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Alert title — does not delete any saved lists, just this pair's level/accent settings</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -9689,27 +9689,27 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>remove_language_confirm_title</t>
+          <t>remove_language_confirm_message</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Remove language?</t>
+          <t>This removes {source} → {target} from your languages. Your saved lists aren't affected.</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>¿Eliminar idioma?</t>
+          <t>Esto elimina {source} → {target} de tus idiomas. Tus listas guardadas no se ven afectadas.</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Supprimer la langue ?</t>
+          <t>Cela supprime {source} → {target} de tes langues. Tes listes enregistrées ne sont pas affectées.</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>Alert title — does not delete any saved lists, just this pair's level/accent settings</t>
+          <t>Template</t>
         </is>
       </c>
     </row>
@@ -9726,27 +9726,27 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>remove_language_confirm_message</t>
+          <t>require_accents_desc</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>This removes {source} → {target} from your languages. Your saved lists aren't affected.</t>
+          <t>Off accepts "cafe" for "café"</t>
         </is>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Esto elimina {source} → {target} de tus idiomas. Tus listas guardadas no se ven afectadas.</t>
+          <t>Desactivado acepta "cafe" en lugar de "café"</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Cela supprime {source} → {target} de tes langues. Tes listes enregistrées ne sont pas affectées.</t>
+          <t>Désactivé accepte "cafe" pour "café"</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>Template</t>
+          <t>Restored — off by default, grading strips accents; app is a reinforcement tool, not a strict teaching tool</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show real error examples and send the focus on Target My Mistakes
Generate Quiz shows the actual "typed → correct" answers behind the
tailored message, passes the AI's focus to question generation only for
Target My Mistakes, and no longer describes ordinary quizzes as
weighted. Also adds localization/generate_translations.py, the script
that builds src/lib/translations/*.ts from ui_strings.csv — it
previously lived only in /tmp and was not in the repo.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G269"/>
+  <dimension ref="A1:G270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9750,6 +9750,43 @@
         </is>
       </c>
     </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>269</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>generate-quiz.tsx</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>insight_examples_label</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>From your last quiz:</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>De tu último cuestionario:</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>De ton dernier quiz :</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Precedes the real 'typed → correct' examples shown under the tailored insight message</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Redesign the feedback display and Generate Quiz layout
- Tailored feedback is now a large card (shared InsightCard) with the
  real mistakes listed under it, on Generate Quiz and Quiz Complete.
  Generate Quiz is titled "Feedback" when it's showing.
- Generate Quiz: word count stays under the list name, question count
  and tense share one row (labelled "No. Questions"), both quiz buttons
  sit together at the bottom, the language pair is centered, and option
  labels are bigger and bolder. The screen scrolls when content is tall.
- Dropdown and the count box share a minimum height so they line up.
- The app sends its UI language with the feedback request so the
  message comes back in it (requires the matching backend change).
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G270"/>
+  <dimension ref="A1:G271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2231,17 +2231,17 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>How many questions?</t>
+          <t>No. Questions</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>¿Cuántas preguntas?</t>
+          <t>N.º de preguntas</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Combien de questions ?</t>
+          <t>Nb de questions</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -9784,6 +9784,43 @@
       <c r="G270" t="inlineStr">
         <is>
           <t>Precedes the real 'typed → correct' examples shown under the tailored insight message</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>270</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>generate-quiz.tsx</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>feedback_title</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Feedback</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Commentaires</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Screen title used instead of Generate Quiz when the tailored feedback card is showing</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add animations, quiz-flow polish, and fix resumed-quiz score
- Press-scale buttons, animated progress bar (bigger while generating),
  dropdown sheet slide, screen transitions, splash fade-in
- Answer feedback animation, question slide-in, score count-up, confetti
  at 90%+, real generation progress
- List/word/quiz row stagger and delete animations, onboarding slides
- Return key submits quiz answers; keyboard-aware quiz screen
- Resuming a quiz carries earlier correct answers into the score
- Quiz results back button returns to where you came from
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G271"/>
+  <dimension ref="A1:G272"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -483,8 +483,6 @@
           <t>LangReps</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Proper name — may stay untranslated</t>
@@ -522,7 +520,6 @@
           <t>Crée une liste de vocabulaire, puis laisse l'IA générer un quiz adaptatif pour toi.</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -555,7 +552,6 @@
           <t>Paramètres</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -588,7 +584,6 @@
           <t>Se déconnecter</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -658,7 +653,6 @@
           <t>Se connecter / S'inscrire</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -728,7 +722,6 @@
           <t>Ajouter des mots manuellement</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -761,7 +754,6 @@
           <t>Coller une liste de vocabulaire</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -794,7 +786,6 @@
           <t>Importer un fichier</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -827,7 +818,6 @@
           <t>Importer une photo</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -860,7 +850,6 @@
           <t>Mes listes</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -893,7 +882,6 @@
           <t>Mes quiz</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1148,7 +1136,6 @@
           <t>E-mail</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1181,7 +1168,6 @@
           <t>Mot de passe</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1214,7 +1200,6 @@
           <t>Veuillez patienter…</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1247,7 +1232,6 @@
           <t>Pas de compte ? Inscris-toi</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1280,7 +1264,6 @@
           <t>Tu as déjà un compte ? Connecte-toi</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1313,7 +1296,6 @@
           <t>Vérifie tes e-mails pour confirmer, puis connecte-toi ci-dessous.</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1346,7 +1328,6 @@
           <t>Compte créé — connecte-toi ci-dessous.</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1453,7 +1434,6 @@
           <t>Coller une liste de vocabulaire</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1523,7 +1503,6 @@
           <t>Colle ici ta liste de vocabulaire</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1630,7 +1609,6 @@
           <t>Une erreur s'est produite lors de l'analyse de ce texte.</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1663,7 +1641,6 @@
           <t>Importer un fichier</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1696,7 +1673,6 @@
           <t>Un fichier texte brut ou CSV, une paire par ligne — une tabulation, "-&gt;", ":", ou un symbole similaire entre chaque mot et sa traduction.</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1729,7 +1705,6 @@
           <t>Choisir un fichier</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1799,7 +1774,6 @@
           <t>Une erreur s'est produite lors de l'analyse de ce fichier.</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1832,7 +1806,6 @@
           <t>Importer une photo</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1902,7 +1875,6 @@
           <t>Prendre une photo</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1935,7 +1907,6 @@
           <t>Choisir depuis la galerie</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1968,7 +1939,6 @@
           <t>Lecture en cours…</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2001,7 +1971,6 @@
           <t>L'accès à l'appareil photo est nécessaire pour prendre une photo.</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2034,7 +2003,6 @@
           <t>L'accès à la photothèque est nécessaire pour choisir une image.</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2067,7 +2035,6 @@
           <t>Une erreur s'est produite lors de la lecture de cette image.</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2174,7 +2141,6 @@
           <t>Il te faut au moins 3 mots pour générer un quiz.</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2244,7 +2210,6 @@
           <t>Nb de questions</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2277,7 +2242,6 @@
           <t>Temps</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2384,7 +2348,6 @@
           <t>Génération de ton quiz…</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2417,7 +2380,6 @@
           <t>Cibler mes erreurs</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2450,7 +2412,6 @@
           <t>Générer un quiz similaire</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2483,7 +2444,6 @@
           <t>Une erreur s'est produite lors de la génération de ton quiz.</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2516,7 +2476,6 @@
           <t>Mes listes</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2549,7 +2508,6 @@
           <t>Aucune liste enregistrée pour l'instant.</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2619,7 +2577,6 @@
           <t>Supprimer la liste</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2689,7 +2646,6 @@
           <t>Une erreur s'est produite lors du chargement de tes listes.</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2722,7 +2678,6 @@
           <t>Une erreur s'est produite lors du chargement de cette liste.</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2755,7 +2710,6 @@
           <t>Une erreur s'est produite lors de la suppression de cette liste.</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2788,7 +2742,6 @@
           <t>Mes quiz</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2821,7 +2774,6 @@
           <t>Aucun quiz en cours.</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2854,7 +2806,6 @@
           <t>Quiz en cours</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2924,7 +2875,6 @@
           <t>Supprimer le quiz</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2994,7 +2944,6 @@
           <t>Une erreur s'est produite lors du chargement de tes quiz.</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3027,7 +2976,6 @@
           <t>Une erreur s'est produite lors de la suppression de ce quiz.</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3097,7 +3045,6 @@
           <t>Aucun quiz terminé pour l'instant.</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3167,7 +3114,6 @@
           <t>Une erreur s'est produite lors du chargement de l'historique du quiz.</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3200,7 +3146,6 @@
           <t>Paramètres</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3233,7 +3178,6 @@
           <t>Supprimer automatiquement les quiz terminés après 30 jours</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3266,7 +3210,6 @@
           <t>Quiz adaptatifs — retour sur les schémas qui te posent des difficultés, avec la possibilité de les cibler</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3299,7 +3242,6 @@
           <t>Ta réponse</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3332,7 +3274,6 @@
           <t>Valider</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3365,7 +3306,6 @@
           <t>Passer cette question</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3398,7 +3338,6 @@
           <t>Masquer la liste de mots</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3431,7 +3370,6 @@
           <t>Bloqué ? Consulte la liste de mots</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3501,7 +3439,6 @@
           <t>C'est correct !</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3571,7 +3508,6 @@
           <t>Terminer le quiz</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3604,7 +3540,6 @@
           <t>Question suivante</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3637,7 +3572,6 @@
           <t>Quiz terminé !</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3707,7 +3641,6 @@
           <t>Retour à l'accueil</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3740,7 +3673,6 @@
           <t>Annuler le dernier</t>
         </is>
       </c>
-      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3773,7 +3705,6 @@
           <t>Vider la liste</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3806,7 +3737,6 @@
           <t>Aucun mot ajouté pour l'instant.</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3839,7 +3769,6 @@
           <t>Nom de la liste (l'enregistrement la met à jour)</t>
         </is>
       </c>
-      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3872,7 +3801,6 @@
           <t>Nom de la liste</t>
         </is>
       </c>
-      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3905,7 +3833,6 @@
           <t>Enregistrement…</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3938,7 +3865,6 @@
           <t>Enregistrer la liste</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3971,7 +3897,6 @@
           <t>Enregistré !</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4004,7 +3929,6 @@
           <t>Une erreur s'est produite lors de l'enregistrement.</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4370,7 +4294,6 @@
           <t>Tu es en pleine lancée — tes scores récents sont bien au-dessus de ton point de départ.</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4403,7 +4326,6 @@
           <t>Gros bond dans tes scores dernièrement. Continue comme ça, quoi que tu fasses.</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4436,7 +4358,6 @@
           <t>Ta précision a beaucoup augmenté récemment — cette liste porte vraiment ses fruits.</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4469,7 +4390,6 @@
           <t>Belle amélioration ici — on voit que tu t'es beaucoup entraîné.</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4539,7 +4459,6 @@
           <t>Bien joué — tes scores augmentent petit à petit.</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4572,7 +4491,6 @@
           <t>Des progrès constants ici. Continue et ça continuera à payer.</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4605,7 +4523,6 @@
           <t>Tu t'améliores un peu à chaque fois que tu fais le quiz sur cette liste.</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4638,7 +4555,6 @@
           <t>Tendance clairement à la hausse — l'entraînement porte ses fruits.</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4708,7 +4624,6 @@
           <t>Tu es régulier sur cette liste — quelques répétitions de plus sur les mots difficiles pourraient te faire progresser.</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4741,7 +4656,6 @@
           <t>Pas beaucoup de changement dernièrement. Ça vaut le coup de voir quels mots précis te posent problème.</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4774,7 +4688,6 @@
           <t>Ça reste stable pour l'instant — essaie de moins t'appuyer sur la liste de mots visible pour vraiment tester ta mémoire.</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4807,7 +4720,6 @@
           <t>Tes scores sont stables. Une petite révision de tes mots les plus faibles pourrait relancer ta progression.</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4877,7 +4789,6 @@
           <t>Une petite baisse dernièrement. Rien de grave, revois juste cette liste quand tu as l'occasion.</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4910,7 +4821,6 @@
           <t>Les scores ont légèrement chuté — ça pourrait valoir le coup de ralentir lors de ta prochaine tentative.</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4943,7 +4853,6 @@
           <t>Une petite baisse récemment. Ça arrive — une courte session de révision devrait aider.</t>
         </is>
       </c>
-      <c r="G132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4976,7 +4885,6 @@
           <t>Tes scores récents sont un peu plus bas qu'avant — un petit rappel serait peut-être utile.</t>
         </is>
       </c>
-      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5046,7 +4954,6 @@
           <t>Une baisse plus importante que d'habitude — cette liste aurait peut-être besoin d'une vraie révision avant ta prochaine tentative.</t>
         </is>
       </c>
-      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5079,7 +4986,6 @@
           <t>Les scores ont pas mal chuté. Ça vaut le coup de revoir la liste depuis le début.</t>
         </is>
       </c>
-      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5112,7 +5018,6 @@
           <t>C'est une chute assez marquée — ralentir et réviser avant de refaire le quiz pourrait aider.</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5145,7 +5050,6 @@
           <t>Une baisse importante ici. Pas de souci, revois juste la liste avant de t'y remettre.</t>
         </is>
       </c>
-      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5168,8 +5072,6 @@
           <t>Various FastAPI HTTPException / Pydantic validation messages surfaced via e.message</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
           <t>Decided: stays English-only — these are dev-facing/edge-case errors (malformed requests, validation failures), not normal user-facing copy</t>
@@ -5207,7 +5109,6 @@
           <t>Listes types</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5240,7 +5141,6 @@
           <t>Ajoute une liste de 50 mots prête à l'emploi pour n'importe quelle paire de langues — ajoutes-en autant que tu veux, quand tu veux.</t>
         </is>
       </c>
-      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5310,7 +5210,6 @@
           <t>Ajouter</t>
         </is>
       </c>
-      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5343,7 +5242,6 @@
           <t>Ajout en cours…</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5413,7 +5311,6 @@
           <t>Une erreur s'est produite lors de l'ajout de cette liste type.</t>
         </is>
       </c>
-      <c r="G146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5446,7 +5343,6 @@
           <t>Passer</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5479,7 +5375,6 @@
           <t>Retour</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5512,7 +5407,6 @@
           <t>Suivant</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5545,7 +5439,6 @@
           <t>Commencer</t>
         </is>
       </c>
-      <c r="G150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5578,7 +5471,6 @@
           <t>Crée ta liste</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5611,7 +5503,6 @@
           <t>Tape des mots, colle une liste, importe un fichier ou prends une photo — l'IA la lit pour toi. Ou commence directement avec quelques listes types déjà prêtes dans Mes listes.</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5644,7 +5535,6 @@
           <t>Entraîne-toi avec des quiz adaptatifs</t>
         </is>
       </c>
-      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5677,7 +5567,6 @@
           <t>L'IA génère de vraies phrases pour te tester — et plus tu t'entraînes, plus elle cible ce qui te pose vraiment des difficultés.</t>
         </is>
       </c>
-      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5710,7 +5599,6 @@
           <t>Suis ta progression</t>
         </is>
       </c>
-      <c r="G155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5743,7 +5631,6 @@
           <t>Regarde tes scores s'améliorer au fil du temps, liste par liste.</t>
         </is>
       </c>
-      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -5813,7 +5700,6 @@
           <t>Trier par</t>
         </is>
       </c>
-      <c r="G158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -5846,7 +5732,6 @@
           <t>Dernier import</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -5879,7 +5764,6 @@
           <t>Nom</t>
         </is>
       </c>
-      <c r="G160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6060,7 +5944,6 @@
           <t>Inscris-toi pour enregistrer tes listes et suivre ta progression au fil du temps</t>
         </is>
       </c>
-      <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6463,7 +6346,6 @@
           <t>Supprimer les listes</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -6496,7 +6378,6 @@
           <t>Supprimer {count} liste(s) ? Cette action est irréversible.</t>
         </is>
       </c>
-      <c r="G177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -6529,7 +6410,6 @@
           <t>{count} en cours</t>
         </is>
       </c>
-      <c r="G178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -6562,7 +6442,6 @@
           <t>Supprimer les quiz</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -6595,7 +6474,6 @@
           <t>Supprimer {count} quiz ? Cette action est irréversible.</t>
         </is>
       </c>
-      <c r="G180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6961,7 +6839,6 @@
           <t>Introductif — mots et phrases de base pour les besoins quotidiens.</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6994,7 +6871,6 @@
           <t>Intermédiaire élémentaire — phrases simples sur des sujets familiers comme la famille et les courses.</t>
         </is>
       </c>
-      <c r="G191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -7027,7 +6903,6 @@
           <t>Niveau seuil — à l'aise dans les situations quotidiennes, les voyages et les sujets courants.</t>
         </is>
       </c>
-      <c r="G192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -7060,7 +6935,6 @@
           <t>Avancé — capable de discuter de sujets généraux et parfois abstraits avec un vocabulaire varié.</t>
         </is>
       </c>
-      <c r="G193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -7093,7 +6967,6 @@
           <t>Autonome — usage fluide et spontané à des fins sociales, académiques ou professionnelles.</t>
         </is>
       </c>
-      <c r="G194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -7126,7 +6999,6 @@
           <t>Maîtrise — fluidité quasi native avec une expression précise et nuancée.</t>
         </is>
       </c>
-      <c r="G195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -7149,8 +7021,6 @@
           <t>LangReps</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
           <t>Animated splash shown on every app launch (not a navigable screen) — proper name, may stay untranslated</t>
@@ -7215,8 +7085,6 @@
           <t>© 2026 MarApps Development</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr"/>
       <c r="G198" t="inlineStr">
         <is>
           <t>Pinned bottom-right corner</t>
@@ -7328,7 +7196,6 @@
           <t>Aucune réponse enregistrée pour ce quiz.</t>
         </is>
       </c>
-      <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -7361,7 +7228,6 @@
           <t>Ta réponse :</t>
         </is>
       </c>
-      <c r="G202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -7468,7 +7334,6 @@
           <t>Une erreur s'est produite lors du chargement des résultats.</t>
         </is>
       </c>
-      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -7538,7 +7403,6 @@
           <t>Vocabulaire — paires de mots simples (noms, adjectifs, etc.), testées telles quelles.</t>
         </is>
       </c>
-      <c r="G207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -7571,7 +7435,6 @@
           <t>Verbe — les infinitifs sont conjugués en contexte lors de la génération du quiz, donc tu es testé sur de vraies formes verbales (ex. « habla ») plutôt que de simplement retenir l'infinitif (« hablar »).</t>
         </is>
       </c>
-      <c r="G208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -7752,7 +7615,6 @@
           <t>Traduire</t>
         </is>
       </c>
-      <c r="G213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -7785,7 +7647,6 @@
           <t>Traduction en cours…</t>
         </is>
       </c>
-      <c r="G214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -7818,7 +7679,6 @@
           <t>Une erreur s'est produite lors de la traduction de ces mots.</t>
         </is>
       </c>
-      <c r="G215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -7999,7 +7859,6 @@
           <t>Une erreur s'est produite lors du renommage.</t>
         </is>
       </c>
-      <c r="G220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -8328,7 +8187,6 @@
           <t>Tu as ajouté des mots qui n'ont pas encore été enregistrés. Si tu quittes maintenant, tu les perdras.</t>
         </is>
       </c>
-      <c r="G229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -8842,7 +8700,6 @@
           <t>Mot de passe oublié ?</t>
         </is>
       </c>
-      <c r="G243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -8875,7 +8732,6 @@
           <t>Mot de passe oublié</t>
         </is>
       </c>
-      <c r="G244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -8945,7 +8801,6 @@
           <t>Entre ton e-mail et nous t'enverrons un lien pour réinitialiser ton mot de passe.</t>
         </is>
       </c>
-      <c r="G246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -8978,7 +8833,6 @@
           <t>Envoi en cours…</t>
         </is>
       </c>
-      <c r="G247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -9011,7 +8865,6 @@
           <t>Envoyer le lien de réinitialisation</t>
         </is>
       </c>
-      <c r="G248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -9044,7 +8897,6 @@
           <t>Réinitialiser le mot de passe</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -9077,7 +8929,6 @@
           <t>Ce lien semble invalide ou expiré. Demande un nouveau lien depuis l'écran de connexion.</t>
         </is>
       </c>
-      <c r="G250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -9110,7 +8961,6 @@
           <t>Définis un nouveau mot de passe</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -9143,7 +8993,6 @@
           <t>Nouveau mot de passe</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -9176,7 +9025,6 @@
           <t>Enregistrer le nouveau mot de passe</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -9246,7 +9094,6 @@
           <t>Supprimer les mots</t>
         </is>
       </c>
-      <c r="G255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -9464,7 +9311,6 @@
           <t>Qu'apprends-tu ?</t>
         </is>
       </c>
-      <c r="G261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -9571,7 +9417,6 @@
           <t>Tes listes de départ sont prêtes — jette un œil dans Mes listes !</t>
         </is>
       </c>
-      <c r="G264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -9604,7 +9449,6 @@
           <t>Ajouter une langue</t>
         </is>
       </c>
-      <c r="G265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -9637,7 +9481,6 @@
           <t>Tu n'as encore ajouté aucune langue — ajoutes-en une ci-dessous pour commencer.</t>
         </is>
       </c>
-      <c r="G266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -9823,6 +9666,37 @@
           <t>Screen title used instead of Generate Quiz when the tailored feedback card is showing</t>
         </is>
       </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>generate-quiz.tsx</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>generating_progress</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Writing questions… {done} of {total}</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Escribiendo preguntas… {done} de {total}</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Rédaction des questions… {done} sur {total}</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix login keyboard, stop language pairs leaking across accounts, redesign Home auth/settings area
- Login screen: dismiss keyboard on outside tap, lift the screen above the
  keyboard so the error message isn't hidden, password field's return key
  submits.
- Language pairs are device-local, not account-bound, which meant a brand
  new account showed a previous account's pairs (and, downstream, its
  auto-generated sample lists) as already there. Clearing local pairs on
  signup stops this without touching logout/login for an existing user.
- Home: signed-in status and Log out now share one row, first. Delete
  Account moved to a new Account section in Settings (rare + destructive
  doesn't belong on the highest-traffic screen; Log out stayed since it's
  low-risk). Settings is now a gear icon in the top-right corner instead
  of a small text link buried in the auth block. App name is bigger.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G272"/>
+  <dimension ref="A1:G273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9696,7 +9696,41 @@
           <t>Rédaction des questions… {done} sur {total}</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>settings.tsx</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>account_section_title</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>Cuenta</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Compte</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Heading above Delete Account, moved here from Home</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rename My Quizzes to Saved Quizzes; add empty state; fix button width on Quiz Complete
- My Quizzes read as 'go here to start a quiz' when it's actually a
  history/resume screen - starting only ever happens from a list. Renamed
  to Saved Quizzes (title + Home button label, all 3 languages) instead
  of colliding with the existing per-list History screen's naming.
- When there's nothing in progress or completed at all, the screen now
  says so plainly and links straight to My Lists (Sample Lists included)
  instead of two bare 'nothing here' sentences with no next step.
- See Full Results and Back to Home on Quiz Complete are now the same
  button style, in a full-width group so they actually match widths
  instead of each shrinking to its own text.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G273"/>
+  <dimension ref="A1:G276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -869,17 +869,17 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>My Quizzes</t>
+          <t>Saved Quizzes</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Mis cuestionarios</t>
+          <t>Cuestionarios guardados</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Mes quiz</t>
+          <t>Quiz enregistrés</t>
         </is>
       </c>
     </row>
@@ -2729,17 +2729,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>My Quizzes</t>
+          <t>Saved Quizzes</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Mis cuestionarios</t>
+          <t>Cuestionarios guardados</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Mes quiz</t>
+          <t>Quiz enregistrés</t>
         </is>
       </c>
     </row>
@@ -9729,6 +9729,101 @@
       <c r="G273" t="inlineStr">
         <is>
           <t>Heading above Delete Account, moved here from Home</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>no_quizzes_yet_title</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>No quizzes yet</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Aún no hay cuestionarios</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Aucun quiz pour l'instant</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>no_quizzes_yet_hint</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Build a list, then generate a quiz from it — it'll show up here.</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Crea una lista y genera un cuestionario a partir de ella; aparecerá aquí.</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Crée une liste, puis génère un quiz à partir de celle-ci — il apparaîtra ici.</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>browse_lists_button</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Browse Your Lists</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Ver tus listas</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Voir tes listes</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Links to My Lists, which also has ready-made Sample Lists</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename Progress to Quiz History; drop the list-name suffix hack; introduce StartQuizOptions and VocabListPayload
- Progress link renamed to Quiz History (all 3 languages) - it opens a
  per-list score-over-time chart, not a place to track generic progress.
- Backend now disambiguates sample lists by name + language pair (see
  language-tutor-api's VocabListMeta commit), so the frontend's
  displayListName()/getListNameSuffix() suffix-stripping hack is gone
  entirely - every list name is used as-is everywhere (rows, delete
  confirmations, rename, list-history nav).
- startQuiz took 6 positional parameters, two added mid-session for
  resuming a session - now one StartQuizOptions object.
- PairsReview's handleSave and handleSaveChanges each built the same
  save-list request object independently - now one shared
  VocabListPayload built by a single buildListPayload() helper.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -2527,17 +2527,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Progress</t>
+          <t>Quiz History</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Progreso</t>
+          <t>Historial de cuestionarios</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Progrès</t>
+          <t>Historique des quiz</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">

</xml_diff>

<commit_message>
Add multi-select tense picker to Generate Quiz
- New MultiSelectDropdown component: an anchored checkbox-list menu that
  stays open until dismissed, for choosing several long-labeled options
  at once (Spanish/French tense names are far too long for a wrapping
  pill row without the field's height becoming unpredictable as
  selections change). Reuses the same anchor/positioning logic as the
  existing single-select Dropdown.
- Generate Quiz's tense field now lets you pick one or more tenses
  instead of one-or-Mixed; Generate is disabled if a Verb list has none
  selected. Saved Quizzes' history badge shows the joined tense labels
  for a session that covered more than one.
- test-data.tsx (dev-only seed screen) updated to the new field name.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G276"/>
+  <dimension ref="A1:G277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9827,6 +9827,41 @@
         </is>
       </c>
     </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>generate-quiz.tsx</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>select_tenses_placeholder</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Select tenses</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Selecciona los tiempos verbales</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Sélectionne les temps</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Multi-select tense field's collapsed placeholder when nothing's picked (shouldn't normally happen — Generate is disabled with none selected)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Intro shows every launch until 'Don't show again'; show real accents on lenient answers
- The intro slides now appear once per app launch until the user ticks
  'Don't show this again' - the only thing that permanently turns them
  off. Skip and Get Started just dismiss it for this launch. An
  in-memory once-per-launch flag keeps Home from redirecting straight
  back into the intro after it closes (it would otherwise loop forever,
  since dismissing no longer marks it permanently seen), and Home falls
  through to the Settings redirect afterward so a first-time logged-in
  user still gets language setup.
- When accent-leniency graded an answer correct but the typed answer
  differs from the real spelling, the feedback now shows the real word
  with just the accented letters colored and underlined - no sentence,
  so a dropped accent isn't silently never learned.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G278"/>
+  <dimension ref="A1:G279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9897,6 +9897,41 @@
         </is>
       </c>
     </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>onboarding.tsx</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>dont_show_again</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Don't show this again</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>No volver a mostrar</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Ne plus afficher</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Checkbox on the intro screens — the only thing that permanently turns the intro off</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Grammar list type and grammar sample lists
Grammar is now a third list type next to Vocab and Verb: a saved
grammar list reloads as Grammar instead of silently becoming Vocab,
My Quizzes shows a Grammar badge, and the list-type info alert
explains it.

The Sample Lists tab is grouped into "Everyday words" and "Grammar
words" and offers three new curated lists (Subject Pronouns,
Conjunctions, Prepositions). Grammar rows show no word count, since
sizes differ by language. English is now offered as a target
(Spanish to English, French to English).

New strings in English, Spanish and French in the CSV and xlsx, with
translations regenerated. The sample-lists hint no longer says
"50-word".

Needs the backend change that adds the grammar categories.
</commit_message>
<xml_diff>
--- a/localization/ui_strings.xlsx
+++ b/localization/ui_strings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G279"/>
+  <dimension ref="A1:G286"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5128,17 +5128,17 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Add a ready-made 50-word list for any language pair — add as many as you want, whenever you want.</t>
+          <t>Add a ready-made list for any language pair — add as many as you want, whenever you want.</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Añade una lista de 50 palabras ya preparada para cualquier par de idiomas — añade tantas como quieras, cuando quieras.</t>
+          <t>Añade una lista ya preparada para cualquier par de idiomas — añade tantas como quieras, cuando quieras.</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Ajoute une liste de 50 mots prête à l'emploi pour n'importe quelle paire de langues — ajoutes-en autant que tu veux, quand tu veux.</t>
+          <t>Ajoute une liste prête à l'emploi pour n'importe quelle paire de langues — ajoutes-en autant que tu veux, quand tu veux.</t>
         </is>
       </c>
     </row>
@@ -9929,6 +9929,251 @@
       <c r="G279" t="inlineStr">
         <is>
           <t>Checkbox on the intro screens — the only thing that permanently turns the intro off</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>sample_category_subject_pronouns</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Subject Pronouns</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>Pronombres de sujeto</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Pronoms sujets</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Grammar sample-list category label</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>sample_category_conjunctions</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Conjunctions</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Conjunciones</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Conjonctions</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>Grammar sample-list category label</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>sample_category_prepositions</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Prepositions</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Preposiciones</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Prépositions</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>Grammar sample-list category label</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>sample_group_everyday</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Everyday words</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Palabras cotidianas</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Mots du quotidien</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Section header on the Sample Lists tab, above the 50-word lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>my-lists.tsx</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>sample_group_grammar</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Grammar words</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Palabras gramaticales</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Mots grammaticaux</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>Section header on the Sample Lists tab, above the grammar-word lists</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>pairs-review.tsx</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>list_type_info_grammar</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Grammar — function words (pronouns, prepositions, conjunctions, etc.), tested in context: each question gives you the sentence the word depends on.</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Gramática — palabras funcionales (pronombres, preposiciones, conjunciones, etc.), evaluadas en contexto: cada pregunta te da la frase de la que depende la palabra.</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Grammaire — mots outils (pronoms, prépositions, conjonctions, etc.), testés en contexte : chaque question te donne la phrase dont dépend le mot.</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>Third line of the list-type info alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>my-quizzes.tsx</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>quiz_type_badge_grammar</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Grammar</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Gramática</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Grammaire</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>Small badge next to the quiz row title</t>
         </is>
       </c>
     </row>

</xml_diff>